<commit_message>
Ronda 12: ROI v02 con Opcion 3 adoptada y hoja de opciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trabajos/mi-proceso/12-roi/Modelo_ROI_Flujo_Credito.xlsx
+++ b/trabajos/mi-proceso/12-roi/Modelo_ROI_Flujo_Credito.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AOCHOA\Documents\Proyecto preaprobado\taller-opencode-bpmn\trabajos\mi-proceso\12-roi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEB19D02-2D66-4C1B-A235-5B70E90F00C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD8BE77C-E5CA-4B5E-9CCA-6F4676A70ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{1C9F3268-D8B7-43FC-ABDA-9EB356B03851}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C1A5622F-C692-4E0F-9B0F-4B3711E0A6ED}"/>
   </bookViews>
   <sheets>
     <sheet name="LEEME" sheetId="1" r:id="rId1"/>
-    <sheet name="Supuestos" sheetId="2" r:id="rId2"/>
-    <sheet name="Conteos" sheetId="3" r:id="rId3"/>
-    <sheet name="ROI" sheetId="4" r:id="rId4"/>
-    <sheet name="FlujoMensual" sheetId="5" r:id="rId5"/>
+    <sheet name="Opciones" sheetId="2" r:id="rId2"/>
+    <sheet name="ROI" sheetId="3" r:id="rId3"/>
+    <sheet name="Supuestos" sheetId="4" r:id="rId4"/>
+    <sheet name="Conteos" sheetId="5" r:id="rId5"/>
+    <sheet name="FlujoMensual" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="164">
   <si>
     <t>Modelo de ROI - Flujo de crédito preaprobado Expomóvil (SINTÉTICO)</t>
   </si>
@@ -54,10 +55,16 @@
     <t>Moneda: pesos dominicanos (RD$). Celdas amarillas de la hoja Supuestos = editables.</t>
   </si>
   <si>
-    <t>Caja = menos personal temporal en feria (ROI-4). Las horas liberadas fuera de feria son CAPACIDAD, no ahorro en caja.</t>
-  </si>
-  <si>
-    <t>ROI año 1 = (beneficio en caja - opex - inversión) / (opex + inversión). Opex = mensajero + mantenimiento.</t>
+    <t>MODELO ADOPTADO = Opción 3 (ronda 12): versión mínima del portal sobre Camunda, cliente entrega originales en sucursal (sin mensajero) y el tiempo liberado fuera de feria se convierte en caja (no reponer puestos).</t>
+  </si>
+  <si>
+    <t>Hoja Opciones: compara el modelo original con las opciones 1, 2 y 3 (escenario base). Hojas ROI y FlujoMensual: modelo adoptado.</t>
+  </si>
+  <si>
+    <t>Caja = menos personal temporal en feria (ROI-4) + tiempo liberado convertido en caja (% editable en Supuestos, fila 24).</t>
+  </si>
+  <si>
+    <t>ROI año 1 = (beneficio en caja - opex - inversión) / (opex + inversión). Opex = mensajero (si aplica) + mantenimiento.</t>
   </si>
   <si>
     <t>Beneficio NO incluido: créditos que dejan de perderse por vencimiento (ver ROI, fila 28). Falta el margen por crédito.</t>
@@ -159,16 +166,16 @@
     <t>RD$/recogida</t>
   </si>
   <si>
-    <t>SUPUESTO S-2</t>
-  </si>
-  <si>
-    <t>Inversión inicial: portal + validación automática</t>
+    <t>SUPUESTO S-2 (solo si hay mensajero, fila 23)</t>
+  </si>
+  <si>
+    <t>Inversión inicial: versión mínima del portal sobre Camunda</t>
   </si>
   <si>
     <t>RD$</t>
   </si>
   <si>
-    <t>SUPUESTO S-3 (desarrollo de IT del banco)</t>
+    <t>SUPUESTO S-3b (Opción 3, ronda 12)</t>
   </si>
   <si>
     <t>Mantenimiento anual (% de la inversión)</t>
@@ -177,7 +184,19 @@
     <t>%</t>
   </si>
   <si>
-    <t>SUPUESTO S-4</t>
+    <t>SUPUESTO S-4b (Opción 3)</t>
+  </si>
+  <si>
+    <t>¿Mensajero a domicilio? (1 = sí, 0 = cliente entrega en sucursal)</t>
+  </si>
+  <si>
+    <t>Decisión Opción 1 (ronda 12)</t>
+  </si>
+  <si>
+    <t>% del tiempo liberado fuera de feria que se convierte en caja</t>
+  </si>
+  <si>
+    <t>Decisión Opción 2 (ronda 12): no reponer puestos; SUPUESTO S-5 en conservador</t>
   </si>
   <si>
     <t>Horas de trabajo por ejecución de cada actividad</t>
@@ -291,7 +310,7 @@
     <t>2026-12</t>
   </si>
   <si>
-    <t>ROI del TO-BE: tres escenarios (año 1)</t>
+    <t>ROI del modelo adoptado (Opción 3): tres escenarios de sensibilidad (año 1)</t>
   </si>
   <si>
     <t>Concepto</t>
@@ -348,10 +367,16 @@
     <t>Capacidad, no caja</t>
   </si>
   <si>
-    <t>Valor de la capacidad liberada (NO es caja)</t>
-  </si>
-  <si>
-    <t>Solo referencia</t>
+    <t>Valor del tiempo liberado fuera de feria</t>
+  </si>
+  <si>
+    <t>Horas liberadas x costo hora</t>
+  </si>
+  <si>
+    <t>AHORRO EN CAJA: tiempo liberado convertido (no reponer puestos)</t>
+  </si>
+  <si>
+    <t>Opción 2: valor x % convertido</t>
   </si>
   <si>
     <t>Recogidas a domicilio</t>
@@ -360,10 +385,13 @@
     <t>recogidas/año</t>
   </si>
   <si>
+    <t>TB_ACT_RECOGER; 0 si el cliente entrega en sucursal (Opción 1)</t>
+  </si>
+  <si>
     <t>Costo del mensajero certificado</t>
   </si>
   <si>
-    <t>Costo nuevo del TO-BE</t>
+    <t>Recogidas x costo por recogida</t>
   </si>
   <si>
     <t>Mantenimiento del portal</t>
@@ -375,13 +403,22 @@
     <t>Mensajero + mantenimiento</t>
   </si>
   <si>
-    <t>Inversión inicial</t>
+    <t>Inversión inicial (versión mínima)</t>
+  </si>
+  <si>
+    <t>Opción 3</t>
+  </si>
+  <si>
+    <t>Beneficio total en caja</t>
+  </si>
+  <si>
+    <t>Temporales en feria + tiempo convertido</t>
   </si>
   <si>
     <t>Beneficio neto operativo anual (caja)</t>
   </si>
   <si>
-    <t>Ahorro en caja - opex</t>
+    <t>Beneficio en caja - opex</t>
   </si>
   <si>
     <t>ROI año 1 (caja)</t>
@@ -399,10 +436,10 @@
     <t>Inversión / beneficio neto mensual</t>
   </si>
   <si>
-    <t>ROI año 1 si la capacidad se monetizara (referencia, NO caja)</t>
-  </si>
-  <si>
-    <t>Solo si se reduce gasto o se produce más</t>
+    <t>ROI año 1 sin convertir el tiempo liberado en caja (referencia)</t>
+  </si>
+  <si>
+    <t>Si no se ejecuta la Opción 2</t>
   </si>
   <si>
     <t>NO INCLUIDO: créditos que dejan de perderse por vencimiento</t>
@@ -414,7 +451,7 @@
     <t>Falta el margen por crédito para monetizarlo</t>
   </si>
   <si>
-    <t>Flujo mensual - escenario BASE (RD$)</t>
+    <t>Flujo mensual - modelo adoptado (Opción 3), escenario BASE (RD$)</t>
   </si>
   <si>
     <t>Horas AS-IS</t>
@@ -426,10 +463,10 @@
     <t>Horas ahorradas</t>
   </si>
   <si>
-    <t>Ahorro en caja (feria)</t>
-  </si>
-  <si>
-    <t>Capacidad (no caja)</t>
+    <t>Ahorro temporales (feria)</t>
+  </si>
+  <si>
+    <t>Tiempo convertido en caja</t>
   </si>
   <si>
     <t>Mensajero</t>
@@ -448,6 +485,57 @@
   </si>
   <si>
     <t>inversión</t>
+  </si>
+  <si>
+    <t>Opciones para subir el ROI (escenario base, año 1) - ronda 12</t>
+  </si>
+  <si>
+    <t>Modelo original</t>
+  </si>
+  <si>
+    <t>Opción 1: sin mensajero</t>
+  </si>
+  <si>
+    <t>Opción 2: + tiempo en caja</t>
+  </si>
+  <si>
+    <t>Opción 3: + versión mínima (ADOPTADA)</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>Inversión inicial (RD$)</t>
+  </si>
+  <si>
+    <t>Portal completo vs versión mínima sobre Camunda</t>
+  </si>
+  <si>
+    <t>¿Mensajero a domicilio? (1/0)</t>
+  </si>
+  <si>
+    <t>Opción 1: el cliente entrega los originales en sucursal o en la feria</t>
+  </si>
+  <si>
+    <t>% del tiempo liberado que se convierte en caja</t>
+  </si>
+  <si>
+    <t>Opción 2: no reponer ~2,7 puestos fuera de feria</t>
+  </si>
+  <si>
+    <t>Ahorro temporales en feria</t>
+  </si>
+  <si>
+    <t>Tiempo liberado convertido en caja</t>
+  </si>
+  <si>
+    <t>Opex</t>
+  </si>
+  <si>
+    <t>Beneficio neto anual (caja)</t>
+  </si>
+  <si>
+    <t>La columna de la Opción 3 toma sus valores de la hoja Supuestos (columna Base). Las columnas B a D son editables.</t>
   </si>
 </sst>
 </file>
@@ -485,7 +573,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,6 +592,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -517,12 +611,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -534,6 +629,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -867,8 +969,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15E9E1B-3773-4317-B696-83FC9A60A059}">
-  <dimension ref="A1:A8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{526EB361-1192-44C4-89D9-02E4374A6B3C}">
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="120.77734375" customWidth="1"/>
@@ -909,376 +1011,335 @@
         <v>6</v>
       </c>
     </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C529142-D840-43BD-AAD5-64C5AA9AD3B6}">
-  <dimension ref="A1:F22"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B58626E5-5D32-4FF2-95B5-8EFF4BC8CAF8}">
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="50.77734375" customWidth="1"/>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.77734375" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="53.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>148</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>10</v>
+        <v>149</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
+        <v>150</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>151</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>13</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="5">
-        <v>29988</v>
-      </c>
-      <c r="D4" s="5">
-        <v>29988</v>
-      </c>
-      <c r="E4" s="5">
-        <v>29988</v>
+        <v>153</v>
+      </c>
+      <c r="B4" s="6">
+        <v>3500000</v>
+      </c>
+      <c r="C4" s="6">
+        <v>3500000</v>
+      </c>
+      <c r="D4" s="6">
+        <v>3500000</v>
+      </c>
+      <c r="E4" s="18">
+        <f>Supuestos!D20</f>
+        <v>1000000</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="4">
-        <v>1.25</v>
-      </c>
-      <c r="D5" s="4">
-        <v>1.25</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1.25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>19</v>
+        <v>44</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="C5" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="D5" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="E5" s="19">
+        <f>Supuestos!D21</f>
+        <v>0.15</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
+        <v>155</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1</v>
       </c>
       <c r="C6" s="4">
-        <v>23.83</v>
+        <v>0</v>
       </c>
       <c r="D6" s="4">
-        <v>23.83</v>
-      </c>
-      <c r="E6" s="4">
-        <v>23.83</v>
+        <v>0</v>
+      </c>
+      <c r="E6" s="20">
+        <f>Supuestos!D23</f>
+        <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>22</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="4">
-        <v>8</v>
-      </c>
-      <c r="D7" s="4">
-        <v>8</v>
-      </c>
-      <c r="E7" s="4">
-        <v>8</v>
+        <v>157</v>
+      </c>
+      <c r="B7" s="8">
+        <v>0</v>
+      </c>
+      <c r="C7" s="8">
+        <v>0</v>
+      </c>
+      <c r="D7" s="8">
+        <v>1</v>
+      </c>
+      <c r="E7" s="19">
+        <f>Supuestos!D24</f>
+        <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="6">
-        <f>C4*C5/(C6*C7)</f>
-        <v>196.62715065044063</v>
-      </c>
-      <c r="D8" s="6">
-        <f>D4*D5/(D6*D7)</f>
-        <v>196.62715065044063</v>
-      </c>
-      <c r="E8" s="6">
-        <f>E4*E5/(E6*E7)</f>
-        <v>196.62715065044063</v>
-      </c>
-      <c r="F8" t="s">
-        <v>48</v>
+      <c r="E8" s="20"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" s="9">
+        <f>ROI!$D$9</f>
+        <v>351618.50215065043</v>
+      </c>
+      <c r="C9" s="9">
+        <f>ROI!$D$9</f>
+        <v>351618.50215065043</v>
+      </c>
+      <c r="D9" s="9">
+        <f>ROI!$D$9</f>
+        <v>351618.50215065043</v>
+      </c>
+      <c r="E9" s="18">
+        <f>ROI!$D$9</f>
+        <v>351618.50215065043</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>45</v>
+      <c r="A10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B10" s="9">
+        <f>ROI!$D$14*B7</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="9">
+        <f>ROI!$D$14*C7</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="9">
+        <f>ROI!$D$14*D7</f>
+        <v>1022166.2426563156</v>
+      </c>
+      <c r="E10" s="18">
+        <f>ROI!$D$14*E7</f>
+        <v>1022166.2426563156</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="D11" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="E11" s="4">
-        <v>2.25</v>
-      </c>
-      <c r="F11" t="s">
-        <v>28</v>
+      <c r="A11" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="14">
+        <f>B9+B10</f>
+        <v>351618.50215065043</v>
+      </c>
+      <c r="C11" s="14">
+        <f>C9+C10</f>
+        <v>351618.50215065043</v>
+      </c>
+      <c r="D11" s="14">
+        <f>D9+D10</f>
+        <v>1373784.744806966</v>
+      </c>
+      <c r="E11" s="21">
+        <f>E9+E10</f>
+        <v>1373784.744806966</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D12" s="4">
-        <v>1</v>
-      </c>
-      <c r="E12" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="F12" t="s">
-        <v>30</v>
+        <v>141</v>
+      </c>
+      <c r="B12" s="9">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!$D$19*B6</f>
+        <v>1020000</v>
+      </c>
+      <c r="C12" s="9">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!$D$19*C6</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="9">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!$D$19*D6</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="18">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!$D$19*E6</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D13" s="4">
-        <v>1</v>
-      </c>
-      <c r="E13" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="F13" t="s">
-        <v>30</v>
+        <v>142</v>
+      </c>
+      <c r="B13" s="9">
+        <f>B4*B5</f>
+        <v>700000</v>
+      </c>
+      <c r="C13" s="9">
+        <f>C4*C5</f>
+        <v>700000</v>
+      </c>
+      <c r="D13" s="9">
+        <f>D4*D5</f>
+        <v>700000</v>
+      </c>
+      <c r="E13" s="18">
+        <f>E4*E5</f>
+        <v>150000</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="D14" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E14" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="F14" t="s">
-        <v>30</v>
+        <v>161</v>
+      </c>
+      <c r="B14" s="9">
+        <f>B12+B13</f>
+        <v>1720000</v>
+      </c>
+      <c r="C14" s="9">
+        <f>C12+C13</f>
+        <v>700000</v>
+      </c>
+      <c r="D14" s="9">
+        <f>D12+D13</f>
+        <v>700000</v>
+      </c>
+      <c r="E14" s="18">
+        <f>E12+E13</f>
+        <v>150000</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="4">
-        <v>0.125</v>
-      </c>
-      <c r="D15" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="E15" s="4">
-        <v>0.375</v>
-      </c>
-      <c r="F15" t="s">
-        <v>30</v>
+      <c r="A15" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" s="14">
+        <f>B11-B14</f>
+        <v>-1368381.4978493496</v>
+      </c>
+      <c r="C15" s="14">
+        <f>C11-C14</f>
+        <v>-348381.49784934957</v>
+      </c>
+      <c r="D15" s="14">
+        <f>D11-D14</f>
+        <v>673784.74480696605</v>
+      </c>
+      <c r="E15" s="21">
+        <f>E11-E14</f>
+        <v>1223784.744806966</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D16" s="4">
-        <v>1</v>
-      </c>
-      <c r="E16" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="F16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D17" s="4">
-        <v>1</v>
-      </c>
-      <c r="E17" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="F17" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="15">
+        <f>(B11-B14-B4)/(B14+B4)</f>
+        <v>-0.93264013368761489</v>
+      </c>
+      <c r="C16" s="15">
+        <f>(C11-C14-C4)/(C14+C4)</f>
+        <v>-0.91628130901174987</v>
+      </c>
+      <c r="D16" s="15">
+        <f>(D11-D14-D4)/(D14+D4)</f>
+        <v>-0.67290839409357961</v>
+      </c>
+      <c r="E16" s="22">
+        <f>(E11-E14-E4)/(E14+E4)</f>
+        <v>0.19459543026692699</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="16" t="str">
+        <f>IF(B15&gt;0,B4/(B15/12),"No se recupera")</f>
+        <v>No se recupera</v>
+      </c>
+      <c r="C17" s="16" t="str">
+        <f>IF(C15&gt;0,C4/(C15/12),"No se recupera")</f>
+        <v>No se recupera</v>
+      </c>
+      <c r="D17" s="16">
+        <f>IF(D15&gt;0,D4/(D15/12),"No se recupera")</f>
+        <v>62.334447794647929</v>
+      </c>
+      <c r="E17" s="23">
+        <f>IF(E15&gt;0,E4/(E15/12),"No se recupera")</f>
+        <v>9.8056460099875018</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="5">
-        <v>500</v>
-      </c>
-      <c r="D19" s="5">
-        <v>400</v>
-      </c>
-      <c r="E19" s="5">
-        <v>300</v>
-      </c>
-      <c r="F19" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="5">
-        <v>6000000</v>
-      </c>
-      <c r="D20" s="5">
-        <v>3500000</v>
-      </c>
-      <c r="E20" s="5">
-        <v>2000000</v>
-      </c>
-      <c r="F20" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="7">
-        <v>0.25</v>
-      </c>
-      <c r="D21" s="7">
-        <v>0.2</v>
-      </c>
-      <c r="E21" s="7">
-        <v>0.15</v>
-      </c>
-      <c r="F21" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="8">
-        <f>C20*C21</f>
-        <v>1500000</v>
-      </c>
-      <c r="D22" s="8">
-        <f>D20*D21</f>
-        <v>700000</v>
-      </c>
-      <c r="E22" s="8">
-        <f>E20*E21</f>
-        <v>300000</v>
-      </c>
-      <c r="F22" t="s">
-        <v>48</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -1287,7 +1348,935 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5A5589B-768E-4B54-9945-91114766895F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2875807E-45A2-41EC-A4D0-A62AF59646CD}">
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="58.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="52.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
+        <v>1654.75</v>
+      </c>
+      <c r="D5" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
+        <v>3309.5</v>
+      </c>
+      <c r="E5" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
+        <v>4964.25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
+        <v>760.625</v>
+      </c>
+      <c r="D6" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
+        <v>1521.25</v>
+      </c>
+      <c r="E6" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
+        <v>2281.875</v>
+      </c>
+      <c r="F6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="11">
+        <f>C5-C6</f>
+        <v>894.125</v>
+      </c>
+      <c r="D7" s="11">
+        <f>D5-D6</f>
+        <v>1788.25</v>
+      </c>
+      <c r="E7" s="11">
+        <f>E5-E6</f>
+        <v>2682.375</v>
+      </c>
+      <c r="F7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="12">
+        <f>C7/(Supuestos!C6*Supuestos!C7)</f>
+        <v>4.6901227444397824</v>
+      </c>
+      <c r="D8" s="12">
+        <f>D7/(Supuestos!D6*Supuestos!D7)</f>
+        <v>9.3802454888795648</v>
+      </c>
+      <c r="E8" s="12">
+        <f>E7/(Supuestos!E6*Supuestos!E7)</f>
+        <v>14.070368233319346</v>
+      </c>
+      <c r="F8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="14">
+        <f>C7*Supuestos!C8</f>
+        <v>175809.25107532521</v>
+      </c>
+      <c r="D9" s="14">
+        <f>D7*Supuestos!D8</f>
+        <v>351618.50215065043</v>
+      </c>
+      <c r="E9" s="14">
+        <f>E7*Supuestos!E8</f>
+        <v>527427.75322597567</v>
+      </c>
+      <c r="F9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
+        <v>4903.25</v>
+      </c>
+      <c r="D11" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
+        <v>9806.5</v>
+      </c>
+      <c r="E11" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
+        <v>14709.75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
+        <v>2304</v>
+      </c>
+      <c r="D12" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
+        <v>4608</v>
+      </c>
+      <c r="E12" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
+        <v>6912</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>105</v>
+      </c>
+      <c r="B13" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="11">
+        <f>C11-C12</f>
+        <v>2599.25</v>
+      </c>
+      <c r="D13" s="11">
+        <f>D11-D12</f>
+        <v>5198.5</v>
+      </c>
+      <c r="E13" s="11">
+        <f>E11-E12</f>
+        <v>7797.75</v>
+      </c>
+      <c r="F13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="9">
+        <f>C13*Supuestos!C8</f>
+        <v>511083.12132815778</v>
+      </c>
+      <c r="D14" s="9">
+        <f>D13*Supuestos!D8</f>
+        <v>1022166.2426563156</v>
+      </c>
+      <c r="E14" s="9">
+        <f>E13*Supuestos!E8</f>
+        <v>1533249.3639844733</v>
+      </c>
+      <c r="F14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="14">
+        <f>C14*Supuestos!C24</f>
+        <v>255541.56066407889</v>
+      </c>
+      <c r="D15" s="14">
+        <f>D14*Supuestos!D24</f>
+        <v>1022166.2426563156</v>
+      </c>
+      <c r="E15" s="14">
+        <f>E14*Supuestos!E24</f>
+        <v>1533249.3639844733</v>
+      </c>
+      <c r="F15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!C23</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!D23</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!E23</f>
+        <v>0</v>
+      </c>
+      <c r="F16" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="9">
+        <f>C16*Supuestos!C19</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="9">
+        <f>D16*Supuestos!D19</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="9">
+        <f>E16*Supuestos!E19</f>
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="9">
+        <f>Supuestos!C22</f>
+        <v>300000</v>
+      </c>
+      <c r="D18" s="9">
+        <f>Supuestos!D22</f>
+        <v>150000</v>
+      </c>
+      <c r="E18" s="9">
+        <f>Supuestos!E22</f>
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="9">
+        <f>C17+C18</f>
+        <v>300000</v>
+      </c>
+      <c r="D19" s="9">
+        <f>D17+D18</f>
+        <v>150000</v>
+      </c>
+      <c r="E19" s="9">
+        <f>E17+E18</f>
+        <v>70000</v>
+      </c>
+      <c r="F19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="9">
+        <f>Supuestos!C20</f>
+        <v>1500000</v>
+      </c>
+      <c r="D20" s="9">
+        <f>Supuestos!D20</f>
+        <v>1000000</v>
+      </c>
+      <c r="E20" s="9">
+        <f>Supuestos!E20</f>
+        <v>700000</v>
+      </c>
+      <c r="F20" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="14">
+        <f>C9+C15</f>
+        <v>431350.8117394041</v>
+      </c>
+      <c r="D21" s="14">
+        <f>D9+D15</f>
+        <v>1373784.744806966</v>
+      </c>
+      <c r="E21" s="14">
+        <f>E9+E15</f>
+        <v>2060677.117210449</v>
+      </c>
+      <c r="F21" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="14">
+        <f>C21-C19</f>
+        <v>131350.8117394041</v>
+      </c>
+      <c r="D22" s="14">
+        <f>D21-D19</f>
+        <v>1223784.744806966</v>
+      </c>
+      <c r="E22" s="14">
+        <f>E21-E19</f>
+        <v>1990677.117210449</v>
+      </c>
+      <c r="F22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="15">
+        <f>(C21-C19-C20)/(C19+C20)</f>
+        <v>-0.76036066014477544</v>
+      </c>
+      <c r="D23" s="15">
+        <f>(D21-D19-D20)/(D19+D20)</f>
+        <v>0.19459543026692699</v>
+      </c>
+      <c r="E23" s="15">
+        <f>(E21-E19-E20)/(E19+E20)</f>
+        <v>1.6762040483252585</v>
+      </c>
+      <c r="F23" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" s="16">
+        <f>IF(C22&gt;0,C20/(C22/12),"No se recupera")</f>
+        <v>137.03760000898538</v>
+      </c>
+      <c r="D24" s="16">
+        <f>IF(D22&gt;0,D20/(D22/12),"No se recupera")</f>
+        <v>9.8056460099875018</v>
+      </c>
+      <c r="E24" s="16">
+        <f>IF(E22&gt;0,E20/(E22/12),"No se recupera")</f>
+        <v>4.2196697432132959</v>
+      </c>
+      <c r="F24" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="13">
+        <f>(C9-C19-C20)/(C19+C20)</f>
+        <v>-0.90232819384704155</v>
+      </c>
+      <c r="D26" s="13">
+        <f>(D9-D19-D20)/(D19+D20)</f>
+        <v>-0.69424478073856488</v>
+      </c>
+      <c r="E26" s="13">
+        <f>(E9-E19-E20)/(E19+E20)</f>
+        <v>-0.31502889191431732</v>
+      </c>
+      <c r="F26" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" t="s">
+        <v>133</v>
+      </c>
+      <c r="C28" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
+        <v>153</v>
+      </c>
+      <c r="D28" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
+        <v>153</v>
+      </c>
+      <c r="E28" s="11">
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
+        <v>153</v>
+      </c>
+      <c r="F28" t="s">
+        <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A040D3B-701E-4AF3-A22B-7E58920B8AA2}">
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="50.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="6">
+        <v>29988</v>
+      </c>
+      <c r="D4" s="6">
+        <v>29988</v>
+      </c>
+      <c r="E4" s="6">
+        <v>29988</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1.25</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1.25</v>
+      </c>
+      <c r="E5" s="4">
+        <v>1.25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="4">
+        <v>23.83</v>
+      </c>
+      <c r="D6" s="4">
+        <v>23.83</v>
+      </c>
+      <c r="E6" s="4">
+        <v>23.83</v>
+      </c>
+      <c r="F6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="4">
+        <v>8</v>
+      </c>
+      <c r="D7" s="4">
+        <v>8</v>
+      </c>
+      <c r="E7" s="4">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="7">
+        <f>C4*C5/(C6*C7)</f>
+        <v>196.62715065044063</v>
+      </c>
+      <c r="D8" s="7">
+        <f>D4*D5/(D6*D7)</f>
+        <v>196.62715065044063</v>
+      </c>
+      <c r="E8" s="7">
+        <f>E4*E5/(E6*E7)</f>
+        <v>196.62715065044063</v>
+      </c>
+      <c r="F8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="4">
+        <v>2.25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="4">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="F13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="F14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="F15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D16" s="4">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="F16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="6">
+        <v>500</v>
+      </c>
+      <c r="D19" s="6">
+        <v>400</v>
+      </c>
+      <c r="E19" s="6">
+        <v>300</v>
+      </c>
+      <c r="F19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1500000</v>
+      </c>
+      <c r="D20" s="6">
+        <v>1000000</v>
+      </c>
+      <c r="E20" s="6">
+        <v>700000</v>
+      </c>
+      <c r="F20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="D21" s="8">
+        <v>0.15</v>
+      </c>
+      <c r="E21" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="9">
+        <f>C20*C21</f>
+        <v>300000</v>
+      </c>
+      <c r="D22" s="9">
+        <f>D20*D21</f>
+        <v>150000</v>
+      </c>
+      <c r="E22" s="9">
+        <f>E20*E21</f>
+        <v>70000</v>
+      </c>
+      <c r="F22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="5">
+        <v>36526</v>
+      </c>
+      <c r="C23" s="4">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D24" s="8">
+        <v>1</v>
+      </c>
+      <c r="E24" s="8">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132D3AA9-092C-4E7E-AACB-704C615D5293}">
   <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1307,62 +2296,62 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>66</v>
+      <c r="A4" s="10" t="s">
+        <v>72</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D4">
         <v>286</v>
@@ -1399,14 +2388,14 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>66</v>
+      <c r="A5" s="10" t="s">
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1443,14 +2432,14 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>70</v>
+      <c r="A6" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D6">
         <v>470</v>
@@ -1487,14 +2476,14 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>70</v>
+      <c r="A7" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>82</v>
@@ -1531,14 +2520,14 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>72</v>
+      <c r="A8" s="10" t="s">
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D8">
         <v>286</v>
@@ -1575,14 +2564,14 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>72</v>
+      <c r="A9" s="10" t="s">
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D9">
         <v>37</v>
@@ -1619,14 +2608,14 @@
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" t="s">
         <v>73</v>
       </c>
-      <c r="B10" t="s">
-        <v>67</v>
-      </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D10">
         <v>294</v>
@@ -1663,14 +2652,14 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
         <v>73</v>
       </c>
-      <c r="B11" t="s">
-        <v>67</v>
-      </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D11">
         <v>57</v>
@@ -1707,14 +2696,14 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" t="s">
         <v>74</v>
-      </c>
-      <c r="B12" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" t="s">
-        <v>68</v>
       </c>
       <c r="D12">
         <v>310</v>
@@ -1751,14 +2740,14 @@
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
-        <v>74</v>
+      <c r="A13" s="10" t="s">
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D13">
         <v>45</v>
@@ -1795,14 +2784,14 @@
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
-        <v>75</v>
+      <c r="A14" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D14">
         <v>248</v>
@@ -1839,14 +2828,14 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" t="s">
         <v>75</v>
-      </c>
-      <c r="B15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" t="s">
-        <v>69</v>
       </c>
       <c r="D15">
         <v>45</v>
@@ -1883,14 +2872,14 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>76</v>
+      <c r="A16" s="10" t="s">
+        <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D16">
         <v>319</v>
@@ -1927,14 +2916,14 @@
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>76</v>
+      <c r="A17" s="10" t="s">
+        <v>82</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C17" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D17">
         <v>66</v>
@@ -1971,14 +2960,14 @@
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
-        <v>77</v>
+      <c r="A18" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D18">
         <v>304</v>
@@ -2015,14 +3004,14 @@
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
-        <v>77</v>
+      <c r="A19" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D19">
         <v>44</v>
@@ -2059,14 +3048,14 @@
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
-        <v>78</v>
+      <c r="A20" s="10" t="s">
+        <v>84</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D20">
         <v>321</v>
@@ -2103,14 +3092,14 @@
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>78</v>
+      <c r="A21" s="10" t="s">
+        <v>84</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C21" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D21">
         <v>46</v>
@@ -2147,14 +3136,14 @@
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
-        <v>79</v>
+      <c r="A22" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C22" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D22">
         <v>300</v>
@@ -2191,14 +3180,14 @@
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
-        <v>79</v>
+      <c r="A23" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="B23" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C23" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D23">
         <v>31</v>
@@ -2235,14 +3224,14 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>80</v>
+      <c r="A24" s="10" t="s">
+        <v>86</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D24">
         <v>519</v>
@@ -2279,14 +3268,14 @@
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
-        <v>80</v>
+      <c r="A25" s="10" t="s">
+        <v>86</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D25">
         <v>78</v>
@@ -2323,14 +3312,14 @@
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
-        <v>81</v>
+      <c r="A26" s="10" t="s">
+        <v>87</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C26" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D26">
         <v>275</v>
@@ -2367,14 +3356,14 @@
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="9" t="s">
-        <v>81</v>
+      <c r="A27" s="10" t="s">
+        <v>87</v>
       </c>
       <c r="B27" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C27" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D27">
         <v>45</v>
@@ -2415,555 +3404,88 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF0B9B4E-56B7-4BFC-B408-054FFFC1BC77}">
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="58.77734375" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>1654.75</v>
-      </c>
-      <c r="D5" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>3309.5</v>
-      </c>
-      <c r="E5" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>4964.25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>760.625</v>
-      </c>
-      <c r="D6" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>1521.25</v>
-      </c>
-      <c r="E6" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>2281.875</v>
-      </c>
-      <c r="F6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C7" s="10">
-        <f>C5-C6</f>
-        <v>894.125</v>
-      </c>
-      <c r="D7" s="10">
-        <f>D5-D6</f>
-        <v>1788.25</v>
-      </c>
-      <c r="E7" s="10">
-        <f>E5-E6</f>
-        <v>2682.375</v>
-      </c>
-      <c r="F7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" t="s">
-        <v>93</v>
-      </c>
-      <c r="C8" s="11">
-        <f>C7/(Supuestos!C6*Supuestos!C7)</f>
-        <v>4.6901227444397824</v>
-      </c>
-      <c r="D8" s="11">
-        <f>D7/(Supuestos!D6*Supuestos!D7)</f>
-        <v>9.3802454888795648</v>
-      </c>
-      <c r="E8" s="11">
-        <f>E7/(Supuestos!E6*Supuestos!E7)</f>
-        <v>14.070368233319346</v>
-      </c>
-      <c r="F8" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="13">
-        <f>C7*Supuestos!C8</f>
-        <v>175809.25107532521</v>
-      </c>
-      <c r="D9" s="13">
-        <f>D7*Supuestos!D8</f>
-        <v>351618.50215065043</v>
-      </c>
-      <c r="E9" s="13">
-        <f>E7*Supuestos!E8</f>
-        <v>527427.75322597567</v>
-      </c>
-      <c r="F9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" t="s">
-        <v>86</v>
-      </c>
-      <c r="C11" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>4903.25</v>
-      </c>
-      <c r="D11" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>9806.5</v>
-      </c>
-      <c r="E11" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>14709.75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" t="s">
-        <v>86</v>
-      </c>
-      <c r="C12" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>2304</v>
-      </c>
-      <c r="D12" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>4608</v>
-      </c>
-      <c r="E12" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>6912</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>99</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="10">
-        <f>C11-C12</f>
-        <v>2599.25</v>
-      </c>
-      <c r="D13" s="10">
-        <f>D11-D12</f>
-        <v>5198.5</v>
-      </c>
-      <c r="E13" s="10">
-        <f>E11-E12</f>
-        <v>7797.75</v>
-      </c>
-      <c r="F13" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>101</v>
-      </c>
-      <c r="B14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="8">
-        <f>C13*Supuestos!C8</f>
-        <v>511083.12132815778</v>
-      </c>
-      <c r="D14" s="8">
-        <f>D13*Supuestos!D8</f>
-        <v>1022166.2426563156</v>
-      </c>
-      <c r="E14" s="8">
-        <f>E13*Supuestos!E8</f>
-        <v>1533249.3639844733</v>
-      </c>
-      <c r="F14" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>103</v>
-      </c>
-      <c r="B16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
-        <v>2550</v>
-      </c>
-      <c r="D16" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
-        <v>2550</v>
-      </c>
-      <c r="E16" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
-        <v>2550</v>
-      </c>
-      <c r="F16" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>105</v>
-      </c>
-      <c r="B17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" s="8">
-        <f>C16*Supuestos!C19</f>
-        <v>1275000</v>
-      </c>
-      <c r="D17" s="8">
-        <f>D16*Supuestos!D19</f>
-        <v>1020000</v>
-      </c>
-      <c r="E17" s="8">
-        <f>E16*Supuestos!E19</f>
-        <v>765000</v>
-      </c>
-      <c r="F17" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>107</v>
-      </c>
-      <c r="B18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="8">
-        <f>Supuestos!C22</f>
-        <v>1500000</v>
-      </c>
-      <c r="D18" s="8">
-        <f>Supuestos!D22</f>
-        <v>700000</v>
-      </c>
-      <c r="E18" s="8">
-        <f>Supuestos!E22</f>
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>108</v>
-      </c>
-      <c r="B19" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="8">
-        <f>C17+C18</f>
-        <v>2775000</v>
-      </c>
-      <c r="D19" s="8">
-        <f>D17+D18</f>
-        <v>1720000</v>
-      </c>
-      <c r="E19" s="8">
-        <f>E17+E18</f>
-        <v>1065000</v>
-      </c>
-      <c r="F19" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>110</v>
-      </c>
-      <c r="B20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="8">
-        <f>Supuestos!C20</f>
-        <v>6000000</v>
-      </c>
-      <c r="D20" s="8">
-        <f>Supuestos!D20</f>
-        <v>3500000</v>
-      </c>
-      <c r="E20" s="8">
-        <f>Supuestos!E20</f>
-        <v>2000000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="13">
-        <f>C9-C19</f>
-        <v>-2599190.7489246749</v>
-      </c>
-      <c r="D22" s="13">
-        <f>D9-D19</f>
-        <v>-1368381.4978493496</v>
-      </c>
-      <c r="E22" s="13">
-        <f>E9-E19</f>
-        <v>-537572.24677402433</v>
-      </c>
-      <c r="F22" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="14">
-        <f>(C9-C19-C20)/(C19+C20)</f>
-        <v>-0.97996475771221359</v>
-      </c>
-      <c r="D23" s="14">
-        <f>(D9-D19-D20)/(D19+D20)</f>
-        <v>-0.93264013368761489</v>
-      </c>
-      <c r="E23" s="14">
-        <f>(E9-E19-E20)/(E19+E20)</f>
-        <v>-0.82791916697358048</v>
-      </c>
-      <c r="F23" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C24" s="15" t="str">
-        <f>IF(C22&gt;0,C20/(C22/12),"No se recupera")</f>
-        <v>No se recupera</v>
-      </c>
-      <c r="D24" s="15" t="str">
-        <f>IF(D22&gt;0,D20/(D22/12),"No se recupera")</f>
-        <v>No se recupera</v>
-      </c>
-      <c r="E24" s="15" t="str">
-        <f>IF(E22&gt;0,E20/(E22/12),"No se recupera")</f>
-        <v>No se recupera</v>
-      </c>
-      <c r="F24" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>118</v>
-      </c>
-      <c r="B26" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="12">
-        <f>(C9+C14-C19-C20)/(C19+C20)</f>
-        <v>-0.92172166696256608</v>
-      </c>
-      <c r="D26" s="12">
-        <f>(D9+D14-D19-D20)/(D19+D20)</f>
-        <v>-0.7368228458224203</v>
-      </c>
-      <c r="E26" s="12">
-        <f>(E9+E14-E19-E20)/(E19+E20)</f>
-        <v>-0.32767467627717817</v>
-      </c>
-      <c r="F26" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>120</v>
-      </c>
-      <c r="B28" t="s">
-        <v>121</v>
-      </c>
-      <c r="C28" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
-        <v>153</v>
-      </c>
-      <c r="D28" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
-        <v>153</v>
-      </c>
-      <c r="E28" s="10">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
-        <v>153</v>
-      </c>
-      <c r="F28" t="s">
-        <v>122</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B28F0D11-CACE-48BB-9D02-EDC2C34C146F}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8EDECF5-3EB1-452D-AE7C-D1E5DDC2C62D}">
   <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="72.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8">
+        <v>146</v>
+      </c>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9">
         <f>-Supuestos!D20</f>
-        <v>-3500000</v>
-      </c>
-      <c r="K4" s="8">
+        <v>-1000000</v>
+      </c>
+      <c r="K4" s="9">
         <f>J4</f>
-        <v>-3500000</v>
+        <v>-1000000</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="str">
+      <c r="A5" s="10" t="str">
         <f>Conteos!A4</f>
         <v>2026-01</v>
       </c>
@@ -2971,45 +3493,45 @@
         <f>Conteos!B4</f>
         <v>no feria</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="11">
         <f>Conteos!D4*Supuestos!$D$11+Conteos!E4*Supuestos!$D$12+Conteos!F4*Supuestos!$D$13+Conteos!G4*Supuestos!$D$14+Conteos!H4*Supuestos!$D$15+Conteos!I4*Supuestos!$D$16+Conteos!J4*Supuestos!$D$17</f>
         <v>957</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <f>Conteos!D5*Supuestos!$D$11+Conteos!E5*Supuestos!$D$12+Conteos!F5*Supuestos!$D$13+Conteos!G5*Supuestos!$D$14+Conteos!H5*Supuestos!$D$15+Conteos!I5*Supuestos!$D$16+Conteos!J5*Supuestos!$D$17</f>
         <v>439</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="11">
         <f>C5-D5</f>
         <v>518</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="9">
         <f>IF(B5="feria",E5*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="8">
-        <f>IF(B5="no feria",E5*Supuestos!$D$8,0)</f>
+      <c r="G5" s="9">
+        <f>IF(B5="no feria",E5*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>101852.86403692825</v>
       </c>
-      <c r="H5" s="8">
-        <f>Conteos!K5*Supuestos!$D$19</f>
-        <v>70800</v>
-      </c>
-      <c r="I5" s="8">
+      <c r="H5" s="9">
+        <f>Conteos!K5*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J5" s="8">
-        <f>F5-H5-I5</f>
-        <v>-129133.33333333334</v>
-      </c>
-      <c r="K5" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J5" s="9">
+        <f>F5+G5-H5-I5</f>
+        <v>89352.864036928251</v>
+      </c>
+      <c r="K5" s="9">
         <f>K4+J5</f>
-        <v>-3629133.3333333335</v>
+        <v>-910647.13596307172</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="str">
+      <c r="A6" s="10" t="str">
         <f>Conteos!A6</f>
         <v>2026-02</v>
       </c>
@@ -3017,45 +3539,45 @@
         <f>Conteos!B6</f>
         <v>feria</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="11">
         <f>Conteos!D6*Supuestos!$D$11+Conteos!E6*Supuestos!$D$12+Conteos!F6*Supuestos!$D$13+Conteos!G6*Supuestos!$D$14+Conteos!H6*Supuestos!$D$15+Conteos!I6*Supuestos!$D$16+Conteos!J6*Supuestos!$D$17</f>
         <v>1583</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="11">
         <f>Conteos!D7*Supuestos!$D$11+Conteos!E7*Supuestos!$D$12+Conteos!F7*Supuestos!$D$13+Conteos!G7*Supuestos!$D$14+Conteos!H7*Supuestos!$D$15+Conteos!I7*Supuestos!$D$16+Conteos!J7*Supuestos!$D$17</f>
         <v>746.25</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="11">
         <f>C6-D6</f>
         <v>836.75</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="9">
         <f>IF(B6="feria",E6*Supuestos!$D$8,0)</f>
         <v>164527.76830675619</v>
       </c>
-      <c r="G6" s="8">
-        <f>IF(B6="no feria",E6*Supuestos!$D$8,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="8">
-        <f>Conteos!K7*Supuestos!$D$19</f>
-        <v>118000</v>
-      </c>
-      <c r="I6" s="8">
+      <c r="G6" s="9">
+        <f>IF(B6="no feria",E6*Supuestos!$D$8*Supuestos!$D$24,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="9">
+        <f>Conteos!K7*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J6" s="8">
-        <f>F6-H6-I6</f>
-        <v>-11805.565026577147</v>
-      </c>
-      <c r="K6" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J6" s="9">
+        <f>F6+G6-H6-I6</f>
+        <v>152027.76830675619</v>
+      </c>
+      <c r="K6" s="9">
         <f>K5+J6</f>
-        <v>-3640938.8983599106</v>
+        <v>-758619.36765631556</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="str">
+      <c r="A7" s="10" t="str">
         <f>Conteos!A8</f>
         <v>2026-03</v>
       </c>
@@ -3063,45 +3585,45 @@
         <f>Conteos!B8</f>
         <v>no feria</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="11">
         <f>Conteos!D8*Supuestos!$D$11+Conteos!E8*Supuestos!$D$12+Conteos!F8*Supuestos!$D$13+Conteos!G8*Supuestos!$D$14+Conteos!H8*Supuestos!$D$15+Conteos!I8*Supuestos!$D$16+Conteos!J8*Supuestos!$D$17</f>
         <v>955</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="11">
         <f>Conteos!D9*Supuestos!$D$11+Conteos!E9*Supuestos!$D$12+Conteos!F9*Supuestos!$D$13+Conteos!G9*Supuestos!$D$14+Conteos!H9*Supuestos!$D$15+Conteos!I9*Supuestos!$D$16+Conteos!J9*Supuestos!$D$17</f>
         <v>427.5</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="11">
         <f>C7-D7</f>
         <v>527.5</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="9">
         <f>IF(B7="feria",E7*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="8">
-        <f>IF(B7="no feria",E7*Supuestos!$D$8,0)</f>
+      <c r="G7" s="9">
+        <f>IF(B7="no feria",E7*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>103720.82196810743</v>
       </c>
-      <c r="H7" s="8">
-        <f>Conteos!K9*Supuestos!$D$19</f>
-        <v>76000</v>
-      </c>
-      <c r="I7" s="8">
+      <c r="H7" s="9">
+        <f>Conteos!K9*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J7" s="8">
-        <f>F7-H7-I7</f>
-        <v>-134333.33333333334</v>
-      </c>
-      <c r="K7" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J7" s="9">
+        <f>F7+G7-H7-I7</f>
+        <v>91220.821968107426</v>
+      </c>
+      <c r="K7" s="9">
         <f>K6+J7</f>
-        <v>-3775272.2316932441</v>
+        <v>-667398.54568820819</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="str">
+      <c r="A8" s="10" t="str">
         <f>Conteos!A10</f>
         <v>2026-04</v>
       </c>
@@ -3109,45 +3631,45 @@
         <f>Conteos!B10</f>
         <v>no feria</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="11">
         <f>Conteos!D10*Supuestos!$D$11+Conteos!E10*Supuestos!$D$12+Conteos!F10*Supuestos!$D$13+Conteos!G10*Supuestos!$D$14+Conteos!H10*Supuestos!$D$15+Conteos!I10*Supuestos!$D$16+Conteos!J10*Supuestos!$D$17</f>
         <v>971</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="11">
         <f>Conteos!D11*Supuestos!$D$11+Conteos!E11*Supuestos!$D$12+Conteos!F11*Supuestos!$D$13+Conteos!G11*Supuestos!$D$14+Conteos!H11*Supuestos!$D$15+Conteos!I11*Supuestos!$D$16+Conteos!J11*Supuestos!$D$17</f>
         <v>497.5</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="11">
         <f>C8-D8</f>
         <v>473.5</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="9">
         <f>IF(B8="feria",E8*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="8">
-        <f>IF(B8="no feria",E8*Supuestos!$D$8,0)</f>
+      <c r="G8" s="9">
+        <f>IF(B8="no feria",E8*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>93102.955832983644</v>
       </c>
-      <c r="H8" s="8">
-        <f>Conteos!K11*Supuestos!$D$19</f>
-        <v>77200</v>
-      </c>
-      <c r="I8" s="8">
+      <c r="H8" s="9">
+        <f>Conteos!K11*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J8" s="8">
-        <f>F8-H8-I8</f>
-        <v>-135533.33333333334</v>
-      </c>
-      <c r="K8" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J8" s="9">
+        <f>F8+G8-H8-I8</f>
+        <v>80602.955832983644</v>
+      </c>
+      <c r="K8" s="9">
         <f>K7+J8</f>
-        <v>-3910805.5650265776</v>
+        <v>-586795.58985522459</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="str">
+      <c r="A9" s="10" t="str">
         <f>Conteos!A12</f>
         <v>2026-05</v>
       </c>
@@ -3155,45 +3677,45 @@
         <f>Conteos!B12</f>
         <v>no feria</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="11">
         <f>Conteos!D12*Supuestos!$D$11+Conteos!E12*Supuestos!$D$12+Conteos!F12*Supuestos!$D$13+Conteos!G12*Supuestos!$D$14+Conteos!H12*Supuestos!$D$15+Conteos!I12*Supuestos!$D$16+Conteos!J12*Supuestos!$D$17</f>
         <v>1019</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="11">
         <f>Conteos!D13*Supuestos!$D$11+Conteos!E13*Supuestos!$D$12+Conteos!F13*Supuestos!$D$13+Conteos!G13*Supuestos!$D$14+Conteos!H13*Supuestos!$D$15+Conteos!I13*Supuestos!$D$16+Conteos!J13*Supuestos!$D$17</f>
         <v>472.5</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="11">
         <f>C9-D9</f>
         <v>546.5</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="9">
         <f>IF(B9="feria",E9*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="8">
-        <f>IF(B9="no feria",E9*Supuestos!$D$8,0)</f>
+      <c r="G9" s="9">
+        <f>IF(B9="no feria",E9*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>107456.73783046581</v>
       </c>
-      <c r="H9" s="8">
-        <f>Conteos!K13*Supuestos!$D$19</f>
-        <v>81600</v>
-      </c>
-      <c r="I9" s="8">
+      <c r="H9" s="9">
+        <f>Conteos!K13*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J9" s="8">
-        <f>F9-H9-I9</f>
-        <v>-139933.33333333334</v>
-      </c>
-      <c r="K9" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J9" s="9">
+        <f>F9+G9-H9-I9</f>
+        <v>94956.737830465805</v>
+      </c>
+      <c r="K9" s="9">
         <f>K8+J9</f>
-        <v>-4050738.8983599111</v>
+        <v>-491838.85202475882</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="str">
+      <c r="A10" s="10" t="str">
         <f>Conteos!A14</f>
         <v>2026-06</v>
       </c>
@@ -3201,45 +3723,45 @@
         <f>Conteos!B14</f>
         <v>no feria</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="11">
         <f>Conteos!D14*Supuestos!$D$11+Conteos!E14*Supuestos!$D$12+Conteos!F14*Supuestos!$D$13+Conteos!G14*Supuestos!$D$14+Conteos!H14*Supuestos!$D$15+Conteos!I14*Supuestos!$D$16+Conteos!J14*Supuestos!$D$17</f>
         <v>810</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="11">
         <f>Conteos!D15*Supuestos!$D$11+Conteos!E15*Supuestos!$D$12+Conteos!F15*Supuestos!$D$13+Conteos!G15*Supuestos!$D$14+Conteos!H15*Supuestos!$D$15+Conteos!I15*Supuestos!$D$16+Conteos!J15*Supuestos!$D$17</f>
         <v>420.25</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="11">
         <f>C10-D10</f>
         <v>389.75</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="9">
         <f>IF(B10="feria",E10*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="8">
-        <f>IF(B10="no feria",E10*Supuestos!$D$8,0)</f>
+      <c r="G10" s="9">
+        <f>IF(B10="no feria",E10*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>76635.43196600923</v>
       </c>
-      <c r="H10" s="8">
-        <f>Conteos!K15*Supuestos!$D$19</f>
-        <v>69600</v>
-      </c>
-      <c r="I10" s="8">
+      <c r="H10" s="9">
+        <f>Conteos!K15*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J10" s="8">
-        <f>F10-H10-I10</f>
-        <v>-127933.33333333334</v>
-      </c>
-      <c r="K10" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J10" s="9">
+        <f>F10+G10-H10-I10</f>
+        <v>64135.43196600923</v>
+      </c>
+      <c r="K10" s="9">
         <f>K9+J10</f>
-        <v>-4178672.2316932445</v>
+        <v>-427703.42005874962</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="str">
+      <c r="A11" s="10" t="str">
         <f>Conteos!A16</f>
         <v>2026-07</v>
       </c>
@@ -3247,45 +3769,45 @@
         <f>Conteos!B16</f>
         <v>no feria</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="11">
         <f>Conteos!D16*Supuestos!$D$11+Conteos!E16*Supuestos!$D$12+Conteos!F16*Supuestos!$D$13+Conteos!G16*Supuestos!$D$14+Conteos!H16*Supuestos!$D$15+Conteos!I16*Supuestos!$D$16+Conteos!J16*Supuestos!$D$17</f>
         <v>1068.5</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="11">
         <f>Conteos!D17*Supuestos!$D$11+Conteos!E17*Supuestos!$D$12+Conteos!F17*Supuestos!$D$13+Conteos!G17*Supuestos!$D$14+Conteos!H17*Supuestos!$D$15+Conteos!I17*Supuestos!$D$16+Conteos!J17*Supuestos!$D$17</f>
         <v>532.75</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="11">
         <f>C11-D11</f>
         <v>535.75</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="9">
         <f>IF(B11="feria",E11*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="8">
-        <f>IF(B11="no feria",E11*Supuestos!$D$8,0)</f>
+      <c r="G11" s="9">
+        <f>IF(B11="no feria",E11*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>105342.99596097357</v>
       </c>
-      <c r="H11" s="8">
-        <f>Conteos!K17*Supuestos!$D$19</f>
-        <v>79600</v>
-      </c>
-      <c r="I11" s="8">
+      <c r="H11" s="9">
+        <f>Conteos!K17*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J11" s="8">
-        <f>F11-H11-I11</f>
-        <v>-137933.33333333334</v>
-      </c>
-      <c r="K11" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J11" s="9">
+        <f>F11+G11-H11-I11</f>
+        <v>92842.995960973567</v>
+      </c>
+      <c r="K11" s="9">
         <f>K10+J11</f>
-        <v>-4316605.5650265776</v>
+        <v>-334860.42409777606</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="str">
+      <c r="A12" s="10" t="str">
         <f>Conteos!A18</f>
         <v>2026-08</v>
       </c>
@@ -3293,45 +3815,45 @@
         <f>Conteos!B18</f>
         <v>no feria</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="11">
         <f>Conteos!D18*Supuestos!$D$11+Conteos!E18*Supuestos!$D$12+Conteos!F18*Supuestos!$D$13+Conteos!G18*Supuestos!$D$14+Conteos!H18*Supuestos!$D$15+Conteos!I18*Supuestos!$D$16+Conteos!J18*Supuestos!$D$17</f>
         <v>1018</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="11">
         <f>Conteos!D19*Supuestos!$D$11+Conteos!E19*Supuestos!$D$12+Conteos!F19*Supuestos!$D$13+Conteos!G19*Supuestos!$D$14+Conteos!H19*Supuestos!$D$15+Conteos!I19*Supuestos!$D$16+Conteos!J19*Supuestos!$D$17</f>
         <v>461.75</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="11">
         <f>C12-D12</f>
         <v>556.25</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="9">
         <f>IF(B12="feria",E12*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="8">
-        <f>IF(B12="no feria",E12*Supuestos!$D$8,0)</f>
+      <c r="G12" s="9">
+        <f>IF(B12="no feria",E12*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>109373.8525493076</v>
       </c>
-      <c r="H12" s="8">
-        <f>Conteos!K19*Supuestos!$D$19</f>
-        <v>78400</v>
-      </c>
-      <c r="I12" s="8">
+      <c r="H12" s="9">
+        <f>Conteos!K19*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J12" s="8">
-        <f>F12-H12-I12</f>
-        <v>-136733.33333333334</v>
-      </c>
-      <c r="K12" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J12" s="9">
+        <f>F12+G12-H12-I12</f>
+        <v>96873.852549307601</v>
+      </c>
+      <c r="K12" s="9">
         <f>K11+J12</f>
-        <v>-4453338.8983599106</v>
+        <v>-237986.57154846846</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="str">
+      <c r="A13" s="10" t="str">
         <f>Conteos!A20</f>
         <v>2026-09</v>
       </c>
@@ -3339,45 +3861,45 @@
         <f>Conteos!B20</f>
         <v>no feria</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="11">
         <f>Conteos!D20*Supuestos!$D$11+Conteos!E20*Supuestos!$D$12+Conteos!F20*Supuestos!$D$13+Conteos!G20*Supuestos!$D$14+Conteos!H20*Supuestos!$D$15+Conteos!I20*Supuestos!$D$16+Conteos!J20*Supuestos!$D$17</f>
         <v>1069.5</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="11">
         <f>Conteos!D21*Supuestos!$D$11+Conteos!E21*Supuestos!$D$12+Conteos!F21*Supuestos!$D$13+Conteos!G21*Supuestos!$D$14+Conteos!H21*Supuestos!$D$15+Conteos!I21*Supuestos!$D$16+Conteos!J21*Supuestos!$D$17</f>
         <v>465</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="11">
         <f>C13-D13</f>
         <v>604.5</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="9">
         <f>IF(B13="feria",E13*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="8">
-        <f>IF(B13="no feria",E13*Supuestos!$D$8,0)</f>
+      <c r="G13" s="9">
+        <f>IF(B13="no feria",E13*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>118861.11256819135</v>
       </c>
-      <c r="H13" s="8">
-        <f>Conteos!K21*Supuestos!$D$19</f>
-        <v>79200</v>
-      </c>
-      <c r="I13" s="8">
+      <c r="H13" s="9">
+        <f>Conteos!K21*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J13" s="8">
-        <f>F13-H13-I13</f>
-        <v>-137533.33333333334</v>
-      </c>
-      <c r="K13" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J13" s="9">
+        <f>F13+G13-H13-I13</f>
+        <v>106361.11256819135</v>
+      </c>
+      <c r="K13" s="9">
         <f>K12+J13</f>
-        <v>-4590872.2316932436</v>
+        <v>-131625.45898027712</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="str">
+      <c r="A14" s="10" t="str">
         <f>Conteos!A22</f>
         <v>2026-10</v>
       </c>
@@ -3385,45 +3907,45 @@
         <f>Conteos!B22</f>
         <v>no feria</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="11">
         <f>Conteos!D22*Supuestos!$D$11+Conteos!E22*Supuestos!$D$12+Conteos!F22*Supuestos!$D$13+Conteos!G22*Supuestos!$D$14+Conteos!H22*Supuestos!$D$15+Conteos!I22*Supuestos!$D$16+Conteos!J22*Supuestos!$D$17</f>
         <v>1020</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="11">
         <f>Conteos!D23*Supuestos!$D$11+Conteos!E23*Supuestos!$D$12+Conteos!F23*Supuestos!$D$13+Conteos!G23*Supuestos!$D$14+Conteos!H23*Supuestos!$D$15+Conteos!I23*Supuestos!$D$16+Conteos!J23*Supuestos!$D$17</f>
         <v>431.25</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="11">
         <f>C14-D14</f>
         <v>588.75</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="9">
         <f>IF(B14="feria",E14*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="8">
-        <f>IF(B14="no feria",E14*Supuestos!$D$8,0)</f>
+      <c r="G14" s="9">
+        <f>IF(B14="no feria",E14*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>115764.23494544692</v>
       </c>
-      <c r="H14" s="8">
-        <f>Conteos!K23*Supuestos!$D$19</f>
-        <v>82000</v>
-      </c>
-      <c r="I14" s="8">
+      <c r="H14" s="9">
+        <f>Conteos!K23*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J14" s="8">
-        <f>F14-H14-I14</f>
-        <v>-140333.33333333334</v>
-      </c>
-      <c r="K14" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J14" s="9">
+        <f>F14+G14-H14-I14</f>
+        <v>103264.23494544692</v>
+      </c>
+      <c r="K14" s="9">
         <f>K13+J14</f>
-        <v>-4731205.5650265766</v>
+        <v>-28361.2240348302</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="str">
+      <c r="A15" s="10" t="str">
         <f>Conteos!A24</f>
         <v>2026-11</v>
       </c>
@@ -3431,45 +3953,45 @@
         <f>Conteos!B24</f>
         <v>feria</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="11">
         <f>Conteos!D24*Supuestos!$D$11+Conteos!E24*Supuestos!$D$12+Conteos!F24*Supuestos!$D$13+Conteos!G24*Supuestos!$D$14+Conteos!H24*Supuestos!$D$15+Conteos!I24*Supuestos!$D$16+Conteos!J24*Supuestos!$D$17</f>
         <v>1726.5</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="11">
         <f>Conteos!D25*Supuestos!$D$11+Conteos!E25*Supuestos!$D$12+Conteos!F25*Supuestos!$D$13+Conteos!G25*Supuestos!$D$14+Conteos!H25*Supuestos!$D$15+Conteos!I25*Supuestos!$D$16+Conteos!J25*Supuestos!$D$17</f>
         <v>775</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="11">
         <f>C15-D15</f>
         <v>951.5</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="9">
         <f>IF(B15="feria",E15*Supuestos!$D$8,0)</f>
         <v>187090.73384389427</v>
       </c>
-      <c r="G15" s="8">
-        <f>IF(B15="no feria",E15*Supuestos!$D$8,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="8">
-        <f>Conteos!K25*Supuestos!$D$19</f>
-        <v>130000</v>
-      </c>
-      <c r="I15" s="8">
+      <c r="G15" s="9">
+        <f>IF(B15="no feria",E15*Supuestos!$D$8*Supuestos!$D$24,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="9">
+        <f>Conteos!K25*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J15" s="8">
-        <f>F15-H15-I15</f>
-        <v>-1242.5994894390678</v>
-      </c>
-      <c r="K15" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J15" s="9">
+        <f>F15+G15-H15-I15</f>
+        <v>174590.73384389427</v>
+      </c>
+      <c r="K15" s="9">
         <f>K14+J15</f>
-        <v>-4732448.1645160159</v>
+        <v>146229.50980906407</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="str">
+      <c r="A16" s="10" t="str">
         <f>Conteos!A26</f>
         <v>2026-12</v>
       </c>
@@ -3477,41 +3999,41 @@
         <f>Conteos!B26</f>
         <v>no feria</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="11">
         <f>Conteos!D26*Supuestos!$D$11+Conteos!E26*Supuestos!$D$12+Conteos!F26*Supuestos!$D$13+Conteos!G26*Supuestos!$D$14+Conteos!H26*Supuestos!$D$15+Conteos!I26*Supuestos!$D$16+Conteos!J26*Supuestos!$D$17</f>
         <v>918.5</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="11">
         <f>Conteos!D27*Supuestos!$D$11+Conteos!E27*Supuestos!$D$12+Conteos!F27*Supuestos!$D$13+Conteos!G27*Supuestos!$D$14+Conteos!H27*Supuestos!$D$15+Conteos!I27*Supuestos!$D$16+Conteos!J27*Supuestos!$D$17</f>
         <v>460.5</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="11">
         <f>C16-D16</f>
         <v>458</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="9">
         <f>IF(B16="feria",E16*Supuestos!$D$8,0)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="8">
-        <f>IF(B16="no feria",E16*Supuestos!$D$8,0)</f>
+      <c r="G16" s="9">
+        <f>IF(B16="no feria",E16*Supuestos!$D$8*Supuestos!$D$24,0)</f>
         <v>90055.234997901804</v>
       </c>
-      <c r="H16" s="8">
-        <f>Conteos!K27*Supuestos!$D$19</f>
-        <v>77600</v>
-      </c>
-      <c r="I16" s="8">
+      <c r="H16" s="9">
+        <f>Conteos!K27*Supuestos!$D$19*Supuestos!$D$23</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="9">
         <f>Supuestos!$D$22/12</f>
-        <v>58333.333333333336</v>
-      </c>
-      <c r="J16" s="8">
-        <f>F16-H16-I16</f>
-        <v>-135933.33333333334</v>
-      </c>
-      <c r="K16" s="8">
+        <v>12500</v>
+      </c>
+      <c r="J16" s="9">
+        <f>F16+G16-H16-I16</f>
+        <v>77555.234997901804</v>
+      </c>
+      <c r="K16" s="9">
         <f>K15+J16</f>
-        <v>-4868381.4978493489</v>
+        <v>223784.74480696587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ronda 13: mensajero de un tercero cobrado al cliente (REQ-TOBE-016) y ROI v02 ajustado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trabajos/mi-proceso/12-roi/Modelo_ROI_Flujo_Credito.xlsx
+++ b/trabajos/mi-proceso/12-roi/Modelo_ROI_Flujo_Credito.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AOCHOA\Documents\Proyecto preaprobado\taller-opencode-bpmn\trabajos\mi-proceso\12-roi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD8BE77C-E5CA-4B5E-9CCA-6F4676A70ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C914E26B-4756-4098-8CB1-AD050046AF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C1A5622F-C692-4E0F-9B0F-4B3711E0A6ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1601949E-7C14-41C9-8718-E45E8B4FA2C4}"/>
   </bookViews>
   <sheets>
     <sheet name="LEEME" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="165">
   <si>
     <t>Modelo de ROI - Flujo de crédito preaprobado Expomóvil (SINTÉTICO)</t>
   </si>
@@ -55,7 +55,7 @@
     <t>Moneda: pesos dominicanos (RD$). Celdas amarillas de la hoja Supuestos = editables.</t>
   </si>
   <si>
-    <t>MODELO ADOPTADO = Opción 3 (ronda 12): versión mínima del portal sobre Camunda, cliente entrega originales en sucursal (sin mensajero) y el tiempo liberado fuera de feria se convierte en caja (no reponer puestos).</t>
+    <t>MODELO ADOPTADO = Opción 3 (ronda 12): versión mínima del portal sobre Camunda, mensajero de un tercero cobrado al cliente como comisión (sin costo para el banco) y el tiempo liberado fuera de feria se convierte en caja (no reponer puestos).</t>
   </si>
   <si>
     <t>Hoja Opciones: compara el modelo original con las opciones 1, 2 y 3 (escenario base). Hojas ROI y FlujoMensual: modelo adoptado.</t>
@@ -166,7 +166,7 @@
     <t>RD$/recogida</t>
   </si>
   <si>
-    <t>SUPUESTO S-2 (solo si hay mensajero, fila 23)</t>
+    <t>SUPUESTO S-2 (lo paga el banco solo si fila 23 = 1)</t>
   </si>
   <si>
     <t>Inversión inicial: versión mínima del portal sobre Camunda</t>
@@ -187,10 +187,10 @@
     <t>SUPUESTO S-4b (Opción 3)</t>
   </si>
   <si>
-    <t>¿Mensajero a domicilio? (1 = sí, 0 = cliente entrega en sucursal)</t>
-  </si>
-  <si>
-    <t>Decisión Opción 1 (ronda 12)</t>
+    <t>¿El banco paga el mensajero? (1 = sí, 0 = tercero cobrado al cliente como comisión)</t>
+  </si>
+  <si>
+    <t>Decisión Opción 1 (ronda 13, ROI-7)</t>
   </si>
   <si>
     <t>% del tiempo liberado fuera de feria que se convierte en caja</t>
@@ -385,13 +385,13 @@
     <t>recogidas/año</t>
   </si>
   <si>
-    <t>TB_ACT_RECOGER; 0 si el cliente entrega en sucursal (Opción 1)</t>
-  </si>
-  <si>
-    <t>Costo del mensajero certificado</t>
-  </si>
-  <si>
-    <t>Recogidas x costo por recogida</t>
+    <t>TB_ACT_RECOGER (el mensajero se mantiene)</t>
+  </si>
+  <si>
+    <t>Costo del mensajero para el banco</t>
+  </si>
+  <si>
+    <t>Costo para el banco: 0 si lo paga el cliente como comisión (Opción 1)</t>
   </si>
   <si>
     <t>Mantenimiento del portal</t>
@@ -469,7 +469,7 @@
     <t>Tiempo convertido en caja</t>
   </si>
   <si>
-    <t>Mensajero</t>
+    <t>Mensajero (banco)</t>
   </si>
   <si>
     <t>Mantenimiento</t>
@@ -493,7 +493,7 @@
     <t>Modelo original</t>
   </si>
   <si>
-    <t>Opción 1: sin mensajero</t>
+    <t>Opción 1: mensajero cobrado al cliente</t>
   </si>
   <si>
     <t>Opción 2: + tiempo en caja</t>
@@ -511,10 +511,10 @@
     <t>Portal completo vs versión mínima sobre Camunda</t>
   </si>
   <si>
-    <t>¿Mensajero a domicilio? (1/0)</t>
-  </si>
-  <si>
-    <t>Opción 1: el cliente entrega los originales en sucursal o en la feria</t>
+    <t>¿El banco paga el mensajero? (1/0)</t>
+  </si>
+  <si>
+    <t>Opción 1: lo opera un tercero y se cobra al cliente como comisión del servicio</t>
   </si>
   <si>
     <t>% del tiempo liberado que se convierte en caja</t>
@@ -527,6 +527,9 @@
   </si>
   <si>
     <t>Tiempo liberado convertido en caja</t>
+  </si>
+  <si>
+    <t>Mensajero (costo para el banco)</t>
   </si>
   <si>
     <t>Opex</t>
@@ -969,7 +972,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{526EB361-1192-44C4-89D9-02E4374A6B3C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7253B275-FDB9-4301-B028-8A9558C8F422}">
   <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1027,16 +1030,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B58626E5-5D32-4FF2-95B5-8EFF4BC8CAF8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81388185-1D2F-4836-8309-27AE686D458F}">
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.77734375" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="62.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1213,7 +1216,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="B12" s="9">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!$D$19*B6</f>
@@ -1255,7 +1258,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" s="9">
         <f>B12+B13</f>
@@ -1276,7 +1279,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B15" s="14">
         <f>B11-B14</f>
@@ -1339,7 +1342,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -1348,14 +1351,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2875807E-45A2-41EC-A4D0-A62AF59646CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{311F1BAF-9716-4E9B-8407-AC6D51AEE511}">
   <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58.77734375" customWidth="1"/>
     <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="52.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="55.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1615,16 +1618,16 @@
         <v>112</v>
       </c>
       <c r="C16" s="11">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!C23</f>
-        <v>0</v>
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
+        <v>2550</v>
       </c>
       <c r="D16" s="11">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!D23</f>
-        <v>0</v>
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
+        <v>2550</v>
       </c>
       <c r="E16" s="11">
-        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!E23</f>
-        <v>0</v>
+        <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
+        <v>2550</v>
       </c>
       <c r="F16" t="s">
         <v>113</v>
@@ -1638,15 +1641,15 @@
         <v>56</v>
       </c>
       <c r="C17" s="9">
-        <f>C16*Supuestos!C19</f>
+        <f>C16*Supuestos!C19*Supuestos!C23</f>
         <v>0</v>
       </c>
       <c r="D17" s="9">
-        <f>D16*Supuestos!D19</f>
+        <f>D16*Supuestos!D19*Supuestos!D23</f>
         <v>0</v>
       </c>
       <c r="E17" s="9">
-        <f>E16*Supuestos!E19</f>
+        <f>E16*Supuestos!E19*Supuestos!E23</f>
         <v>0</v>
       </c>
       <c r="F17" t="s">
@@ -1863,7 +1866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A040D3B-701E-4AF3-A22B-7E58920B8AA2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C77556EC-89D4-441E-B433-C1A855725710}">
   <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2276,7 +2279,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132D3AA9-092C-4E7E-AACB-704C615D5293}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEE4A0A0-CCC6-4106-8DE8-63127307EE66}">
   <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3405,7 +3408,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8EDECF5-3EB1-452D-AE7C-D1E5DDC2C62D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CB59B9A-3B10-441F-9DBF-88D23AAD34A8}">
   <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3416,7 +3419,7 @@
     <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Ronda 14: BPMN TO-BE v03 con recordatorios, llamada y carga asistida; datos y ROI regenerados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trabajos/mi-proceso/12-roi/Modelo_ROI_Flujo_Credito.xlsx
+++ b/trabajos/mi-proceso/12-roi/Modelo_ROI_Flujo_Credito.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AOCHOA\Documents\Proyecto preaprobado\taller-opencode-bpmn\trabajos\mi-proceso\12-roi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C914E26B-4756-4098-8CB1-AD050046AF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{396A2F9C-B62B-4A4C-91C6-3A7EA3D07DC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1601949E-7C14-41C9-8718-E45E8B4FA2C4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{654B39BF-4876-4894-B5AF-566591CAB46B}"/>
   </bookViews>
   <sheets>
     <sheet name="LEEME" sheetId="1" r:id="rId1"/>
@@ -972,7 +972,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7253B275-FDB9-4301-B028-8A9558C8F422}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97838C2F-1335-4568-8AFC-E03751D7D805}">
   <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1030,7 +1030,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81388185-1D2F-4836-8309-27AE686D458F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B6CBAD8-B666-4BE0-8762-E4F9235F92DE}">
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1157,19 +1157,19 @@
       </c>
       <c r="B9" s="9">
         <f>ROI!$D$9</f>
-        <v>351618.50215065043</v>
+        <v>335986.64367394045</v>
       </c>
       <c r="C9" s="9">
         <f>ROI!$D$9</f>
-        <v>351618.50215065043</v>
+        <v>335986.64367394045</v>
       </c>
       <c r="D9" s="9">
         <f>ROI!$D$9</f>
-        <v>351618.50215065043</v>
+        <v>335986.64367394045</v>
       </c>
       <c r="E9" s="18">
         <f>ROI!$D$9</f>
-        <v>351618.50215065043</v>
+        <v>335986.64367394045</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1186,11 +1186,11 @@
       </c>
       <c r="D10" s="9">
         <f>ROI!$D$14*D7</f>
-        <v>1022166.2426563156</v>
+        <v>1006190.2866659673</v>
       </c>
       <c r="E10" s="18">
         <f>ROI!$D$14*E7</f>
-        <v>1022166.2426563156</v>
+        <v>1006190.2866659673</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1199,19 +1199,19 @@
       </c>
       <c r="B11" s="14">
         <f>B9+B10</f>
-        <v>351618.50215065043</v>
+        <v>335986.64367394045</v>
       </c>
       <c r="C11" s="14">
         <f>C9+C10</f>
-        <v>351618.50215065043</v>
+        <v>335986.64367394045</v>
       </c>
       <c r="D11" s="14">
         <f>D9+D10</f>
-        <v>1373784.744806966</v>
+        <v>1342176.9303399078</v>
       </c>
       <c r="E11" s="21">
         <f>E9+E10</f>
-        <v>1373784.744806966</v>
+        <v>1342176.9303399078</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B12" s="9">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!$D$19*B6</f>
-        <v>1020000</v>
+        <v>1072800</v>
       </c>
       <c r="C12" s="9">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)*Supuestos!$D$19*C6</f>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="B14" s="9">
         <f>B12+B13</f>
-        <v>1720000</v>
+        <v>1772800</v>
       </c>
       <c r="C14" s="9">
         <f>C12+C13</f>
@@ -1283,19 +1283,19 @@
       </c>
       <c r="B15" s="14">
         <f>B11-B14</f>
-        <v>-1368381.4978493496</v>
+        <v>-1436813.3563260594</v>
       </c>
       <c r="C15" s="14">
         <f>C11-C14</f>
-        <v>-348381.49784934957</v>
+        <v>-364013.35632605955</v>
       </c>
       <c r="D15" s="14">
         <f>D11-D14</f>
-        <v>673784.74480696605</v>
+        <v>642176.93033990776</v>
       </c>
       <c r="E15" s="21">
         <f>E11-E14</f>
-        <v>1223784.744806966</v>
+        <v>1192176.9303399078</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1304,19 +1304,19 @@
       </c>
       <c r="B16" s="15">
         <f>(B11-B14-B4)/(B14+B4)</f>
-        <v>-0.93264013368761489</v>
+        <v>-0.93627927407185163</v>
       </c>
       <c r="C16" s="15">
         <f>(C11-C14-C4)/(C14+C4)</f>
-        <v>-0.91628130901174987</v>
+        <v>-0.92000318007763315</v>
       </c>
       <c r="D16" s="15">
         <f>(D11-D14-D4)/(D14+D4)</f>
-        <v>-0.67290839409357961</v>
+        <v>-0.68043406420478392</v>
       </c>
       <c r="E16" s="22">
         <f>(E11-E14-E4)/(E14+E4)</f>
-        <v>0.19459543026692699</v>
+        <v>0.16711037420861544</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="D17" s="16">
         <f>IF(D15&gt;0,D4/(D15/12),"No se recupera")</f>
-        <v>62.334447794647929</v>
+        <v>65.402536303770944</v>
       </c>
       <c r="E17" s="23">
         <f>IF(E15&gt;0,E4/(E15/12),"No se recupera")</f>
-        <v>9.8056460099875018</v>
+        <v>10.065620038947253</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1351,7 +1351,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{311F1BAF-9716-4E9B-8407-AC6D51AEE511}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41407AB3-0E1C-42D6-BA0D-A06358BE843D}">
   <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1395,15 +1395,15 @@
       </c>
       <c r="C5" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>1654.75</v>
+        <v>1628</v>
       </c>
       <c r="D5" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>3309.5</v>
+        <v>3256</v>
       </c>
       <c r="E5" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>4964.25</v>
+        <v>4884</v>
       </c>
       <c r="F5" t="s">
         <v>93</v>
@@ -1418,15 +1418,15 @@
       </c>
       <c r="C6" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>760.625</v>
+        <v>773.625</v>
       </c>
       <c r="D6" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>1521.25</v>
+        <v>1547.25</v>
       </c>
       <c r="E6" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>2281.875</v>
+        <v>2320.875</v>
       </c>
       <c r="F6" t="s">
         <v>95</v>
@@ -1441,15 +1441,15 @@
       </c>
       <c r="C7" s="11">
         <f>C5-C6</f>
-        <v>894.125</v>
+        <v>854.375</v>
       </c>
       <c r="D7" s="11">
         <f>D5-D6</f>
-        <v>1788.25</v>
+        <v>1708.75</v>
       </c>
       <c r="E7" s="11">
         <f>E5-E6</f>
-        <v>2682.375</v>
+        <v>2563.125</v>
       </c>
       <c r="F7" t="s">
         <v>97</v>
@@ -1464,15 +1464,15 @@
       </c>
       <c r="C8" s="12">
         <f>C7/(Supuestos!C6*Supuestos!C7)</f>
-        <v>4.6901227444397824</v>
+        <v>4.4816145614771301</v>
       </c>
       <c r="D8" s="12">
         <f>D7/(Supuestos!D6*Supuestos!D7)</f>
-        <v>9.3802454888795648</v>
+        <v>8.9632291229542602</v>
       </c>
       <c r="E8" s="12">
         <f>E7/(Supuestos!E6*Supuestos!E7)</f>
-        <v>14.070368233319346</v>
+        <v>13.44484368443139</v>
       </c>
       <c r="F8" t="s">
         <v>100</v>
@@ -1487,15 +1487,15 @@
       </c>
       <c r="C9" s="14">
         <f>C7*Supuestos!C8</f>
-        <v>175809.25107532521</v>
+        <v>167993.32183697022</v>
       </c>
       <c r="D9" s="14">
         <f>D7*Supuestos!D8</f>
-        <v>351618.50215065043</v>
+        <v>335986.64367394045</v>
       </c>
       <c r="E9" s="14">
         <f>E7*Supuestos!E8</f>
-        <v>527427.75322597567</v>
+        <v>503979.96551091061</v>
       </c>
       <c r="F9" t="s">
         <v>102</v>
@@ -1510,15 +1510,15 @@
       </c>
       <c r="C11" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>4903.25</v>
+        <v>4875</v>
       </c>
       <c r="D11" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>9806.5</v>
+        <v>9750</v>
       </c>
       <c r="E11" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>14709.75</v>
+        <v>14625</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1530,15 +1530,15 @@
       </c>
       <c r="C12" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!C$11+Conteos!$E$4:$E$27*Supuestos!C$12+Conteos!$F$4:$F$27*Supuestos!C$13+Conteos!$G$4:$G$27*Supuestos!C$14+Conteos!$H$4:$H$27*Supuestos!C$15+Conteos!$I$4:$I$27*Supuestos!C$16+Conteos!$J$4:$J$27*Supuestos!C$17))</f>
-        <v>2304</v>
+        <v>2316.375</v>
       </c>
       <c r="D12" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!D$11+Conteos!$E$4:$E$27*Supuestos!D$12+Conteos!$F$4:$F$27*Supuestos!D$13+Conteos!$G$4:$G$27*Supuestos!D$14+Conteos!$H$4:$H$27*Supuestos!D$15+Conteos!$I$4:$I$27*Supuestos!D$16+Conteos!$J$4:$J$27*Supuestos!D$17))</f>
-        <v>4608</v>
+        <v>4632.75</v>
       </c>
       <c r="E12" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*(Conteos!$B$4:$B$27="no feria")*(Conteos!$D$4:$D$27*Supuestos!E$11+Conteos!$E$4:$E$27*Supuestos!E$12+Conteos!$F$4:$F$27*Supuestos!E$13+Conteos!$G$4:$G$27*Supuestos!E$14+Conteos!$H$4:$H$27*Supuestos!E$15+Conteos!$I$4:$I$27*Supuestos!E$16+Conteos!$J$4:$J$27*Supuestos!E$17))</f>
-        <v>6912</v>
+        <v>6949.125</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1550,15 +1550,15 @@
       </c>
       <c r="C13" s="11">
         <f>C11-C12</f>
-        <v>2599.25</v>
+        <v>2558.625</v>
       </c>
       <c r="D13" s="11">
         <f>D11-D12</f>
-        <v>5198.5</v>
+        <v>5117.25</v>
       </c>
       <c r="E13" s="11">
         <f>E11-E12</f>
-        <v>7797.75</v>
+        <v>7675.875</v>
       </c>
       <c r="F13" t="s">
         <v>106</v>
@@ -1573,15 +1573,15 @@
       </c>
       <c r="C14" s="9">
         <f>C13*Supuestos!C8</f>
-        <v>511083.12132815778</v>
+        <v>503095.14333298366</v>
       </c>
       <c r="D14" s="9">
         <f>D13*Supuestos!D8</f>
-        <v>1022166.2426563156</v>
+        <v>1006190.2866659673</v>
       </c>
       <c r="E14" s="9">
         <f>E13*Supuestos!E8</f>
-        <v>1533249.3639844733</v>
+        <v>1509285.429998951</v>
       </c>
       <c r="F14" t="s">
         <v>108</v>
@@ -1596,15 +1596,15 @@
       </c>
       <c r="C15" s="14">
         <f>C14*Supuestos!C24</f>
-        <v>255541.56066407889</v>
+        <v>251547.57166649183</v>
       </c>
       <c r="D15" s="14">
         <f>D14*Supuestos!D24</f>
-        <v>1022166.2426563156</v>
+        <v>1006190.2866659673</v>
       </c>
       <c r="E15" s="14">
         <f>E14*Supuestos!E24</f>
-        <v>1533249.3639844733</v>
+        <v>1509285.429998951</v>
       </c>
       <c r="F15" t="s">
         <v>110</v>
@@ -1619,15 +1619,15 @@
       </c>
       <c r="C16" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
-        <v>2550</v>
+        <v>2682</v>
       </c>
       <c r="D16" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
-        <v>2550</v>
+        <v>2682</v>
       </c>
       <c r="E16" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$K$4:$K$27)</f>
-        <v>2550</v>
+        <v>2682</v>
       </c>
       <c r="F16" t="s">
         <v>113</v>
@@ -1731,15 +1731,15 @@
       </c>
       <c r="C21" s="14">
         <f>C9+C15</f>
-        <v>431350.8117394041</v>
+        <v>419540.89350346208</v>
       </c>
       <c r="D21" s="14">
         <f>D9+D15</f>
-        <v>1373784.744806966</v>
+        <v>1342176.9303399078</v>
       </c>
       <c r="E21" s="14">
         <f>E9+E15</f>
-        <v>2060677.117210449</v>
+        <v>2013265.3955098616</v>
       </c>
       <c r="F21" t="s">
         <v>122</v>
@@ -1754,15 +1754,15 @@
       </c>
       <c r="C22" s="14">
         <f>C21-C19</f>
-        <v>131350.8117394041</v>
+        <v>119540.89350346208</v>
       </c>
       <c r="D22" s="14">
         <f>D21-D19</f>
-        <v>1223784.744806966</v>
+        <v>1192176.9303399078</v>
       </c>
       <c r="E22" s="14">
         <f>E21-E19</f>
-        <v>1990677.117210449</v>
+        <v>1943265.3955098616</v>
       </c>
       <c r="F22" t="s">
         <v>124</v>
@@ -1777,15 +1777,15 @@
       </c>
       <c r="C23" s="15">
         <f>(C21-C19-C20)/(C19+C20)</f>
-        <v>-0.76036066014477544</v>
+        <v>-0.76692172583141005</v>
       </c>
       <c r="D23" s="15">
         <f>(D21-D19-D20)/(D19+D20)</f>
-        <v>0.19459543026692699</v>
+        <v>0.16711037420861544</v>
       </c>
       <c r="E23" s="15">
         <f>(E21-E19-E20)/(E19+E20)</f>
-        <v>1.6762040483252585</v>
+        <v>1.614630383779041</v>
       </c>
       <c r="F23" t="s">
         <v>126</v>
@@ -1800,15 +1800,15 @@
       </c>
       <c r="C24" s="16">
         <f>IF(C22&gt;0,C20/(C22/12),"No se recupera")</f>
-        <v>137.03760000898538</v>
+        <v>150.57608716534057</v>
       </c>
       <c r="D24" s="16">
         <f>IF(D22&gt;0,D20/(D22/12),"No se recupera")</f>
-        <v>9.8056460099875018</v>
+        <v>10.065620038947253</v>
       </c>
       <c r="E24" s="16">
         <f>IF(E22&gt;0,E20/(E22/12),"No se recupera")</f>
-        <v>4.2196697432132959</v>
+        <v>4.3226210992122676</v>
       </c>
       <c r="F24" t="s">
         <v>129</v>
@@ -1823,15 +1823,15 @@
       </c>
       <c r="C26" s="13">
         <f>(C9-C19-C20)/(C19+C20)</f>
-        <v>-0.90232819384704155</v>
+        <v>-0.90667037675723872</v>
       </c>
       <c r="D26" s="13">
         <f>(D9-D19-D20)/(D19+D20)</f>
-        <v>-0.69424478073856488</v>
+        <v>-0.7078377011530953</v>
       </c>
       <c r="E26" s="13">
         <f>(E9-E19-E20)/(E19+E20)</f>
-        <v>-0.31502889191431732</v>
+        <v>-0.34548056427154467</v>
       </c>
       <c r="F26" t="s">
         <v>131</v>
@@ -1846,15 +1846,15 @@
       </c>
       <c r="C28" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
-        <v>153</v>
+        <v>245</v>
       </c>
       <c r="D28" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
-        <v>153</v>
+        <v>245</v>
       </c>
       <c r="E28" s="11">
         <f>SUMPRODUCT((Conteos!$C$4:$C$27="AS-IS")*Conteos!$M$4:$M$27)-SUMPRODUCT((Conteos!$C$4:$C$27="TO-BE")*Conteos!$M$4:$M$27)</f>
-        <v>153</v>
+        <v>245</v>
       </c>
       <c r="F28" t="s">
         <v>134</v>
@@ -1866,7 +1866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C77556EC-89D4-441E-B433-C1A855725710}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F60780-05D2-4774-9D23-D941924741D6}">
   <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2279,7 +2279,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEE4A0A0-CCC6-4106-8DE8-63127307EE66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68B82A-5D34-4DA8-A33A-65E6950FBB29}">
   <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2357,13 +2357,13 @@
         <v>74</v>
       </c>
       <c r="D4">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E4">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="F4">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -2381,13 +2381,13 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="M4">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="N4">
-        <v>214</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -2404,34 +2404,34 @@
         <v>50</v>
       </c>
       <c r="E5">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F5">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="G5">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="H5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I5">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J5">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="K5">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="L5">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="M5">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="N5">
-        <v>214</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -2445,7 +2445,7 @@
         <v>74</v>
       </c>
       <c r="D6">
-        <v>470</v>
+        <v>487</v>
       </c>
       <c r="E6">
         <v>439</v>
@@ -2469,13 +2469,13 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>378</v>
+        <v>403</v>
       </c>
       <c r="M6">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="N6">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -2489,37 +2489,37 @@
         <v>75</v>
       </c>
       <c r="D7">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E7">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F7">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="G7">
-        <v>308</v>
+        <v>357</v>
       </c>
       <c r="H7">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="I7">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J7">
-        <v>295</v>
+        <v>339</v>
       </c>
       <c r="K7">
-        <v>295</v>
+        <v>339</v>
       </c>
       <c r="L7">
-        <v>378</v>
+        <v>403</v>
       </c>
       <c r="M7">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N7">
-        <v>363</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -2533,13 +2533,13 @@
         <v>74</v>
       </c>
       <c r="D8">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="E8">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="F8">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -2557,13 +2557,13 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="M8">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="N8">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -2577,37 +2577,37 @@
         <v>75</v>
       </c>
       <c r="D9">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E9">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F9">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G9">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="H9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I9">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J9">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="K9">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="L9">
+        <v>239</v>
+      </c>
+      <c r="M9">
+        <v>7</v>
+      </c>
+      <c r="N9">
         <v>232</v>
-      </c>
-      <c r="M9">
-        <v>15</v>
-      </c>
-      <c r="N9">
-        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -2621,13 +2621,13 @@
         <v>74</v>
       </c>
       <c r="D10">
-        <v>294</v>
+        <v>277</v>
       </c>
       <c r="E10">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="F10">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -2645,13 +2645,13 @@
         <v>0</v>
       </c>
       <c r="L10">
-        <v>246</v>
+        <v>225</v>
       </c>
       <c r="M10">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="N10">
-        <v>217</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -2665,37 +2665,37 @@
         <v>75</v>
       </c>
       <c r="D11">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E11">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="F11">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="G11">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H11">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I11">
         <v>9</v>
       </c>
       <c r="J11">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="K11">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="L11">
-        <v>246</v>
+        <v>225</v>
       </c>
       <c r="M11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N11">
-        <v>234</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -2709,13 +2709,13 @@
         <v>74</v>
       </c>
       <c r="D12">
-        <v>310</v>
+        <v>301</v>
       </c>
       <c r="E12">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="F12">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -2733,13 +2733,13 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="M12">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="N12">
-        <v>214</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -2753,37 +2753,37 @@
         <v>75</v>
       </c>
       <c r="D13">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E13">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F13">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="G13">
-        <v>212</v>
+        <v>231</v>
       </c>
       <c r="H13">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="I13">
+        <v>10</v>
+      </c>
+      <c r="J13">
+        <v>217</v>
+      </c>
+      <c r="K13">
+        <v>217</v>
+      </c>
+      <c r="L13">
+        <v>253</v>
+      </c>
+      <c r="M13">
         <v>7</v>
       </c>
-      <c r="J13">
-        <v>204</v>
-      </c>
-      <c r="K13">
-        <v>204</v>
-      </c>
-      <c r="L13">
-        <v>247</v>
-      </c>
-      <c r="M13">
-        <v>10</v>
-      </c>
       <c r="N13">
-        <v>237</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -2797,13 +2797,13 @@
         <v>74</v>
       </c>
       <c r="D14">
-        <v>248</v>
+        <v>282</v>
       </c>
       <c r="E14">
-        <v>219</v>
+        <v>261</v>
       </c>
       <c r="F14">
-        <v>219</v>
+        <v>261</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -2821,13 +2821,13 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="M14">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="N14">
-        <v>191</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -2841,37 +2841,37 @@
         <v>75</v>
       </c>
       <c r="D15">
+        <v>47</v>
+      </c>
+      <c r="E15">
         <v>45</v>
       </c>
-      <c r="E15">
-        <v>38</v>
-      </c>
       <c r="F15">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G15">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="H15">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I15">
         <v>9</v>
       </c>
       <c r="J15">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="K15">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="L15">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="M15">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="N15">
-        <v>202</v>
+        <v>223</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -2885,13 +2885,13 @@
         <v>74</v>
       </c>
       <c r="D16">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="E16">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="F16">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -2909,13 +2909,13 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="M16">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="N16">
-        <v>237</v>
+        <v>227</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
@@ -2929,37 +2929,37 @@
         <v>75</v>
       </c>
       <c r="D17">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="E17">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="F17">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="G17">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="H17">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I17">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J17">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="K17">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="L17">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="M17">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N17">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -2976,10 +2976,10 @@
         <v>304</v>
       </c>
       <c r="E18">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="F18">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -2997,10 +2997,10 @@
         <v>0</v>
       </c>
       <c r="L18">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="M18">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="N18">
         <v>215</v>
@@ -3017,37 +3017,37 @@
         <v>75</v>
       </c>
       <c r="D19">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="E19">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="F19">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="G19">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="H19">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I19">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="J19">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="K19">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="L19">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="M19">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="N19">
-        <v>227</v>
+        <v>242</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -3061,13 +3061,13 @@
         <v>74</v>
       </c>
       <c r="D20">
-        <v>321</v>
+        <v>268</v>
       </c>
       <c r="E20">
-        <v>294</v>
+        <v>250</v>
       </c>
       <c r="F20">
-        <v>294</v>
+        <v>250</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -3085,13 +3085,13 @@
         <v>0</v>
       </c>
       <c r="L20">
-        <v>253</v>
+        <v>215</v>
       </c>
       <c r="M20">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="N20">
-        <v>226</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
@@ -3105,37 +3105,37 @@
         <v>75</v>
       </c>
       <c r="D21">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="E21">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F21">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G21">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="H21">
         <v>12</v>
       </c>
       <c r="I21">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J21">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="K21">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="L21">
-        <v>253</v>
+        <v>215</v>
       </c>
       <c r="M21">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="N21">
-        <v>235</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -3149,13 +3149,13 @@
         <v>74</v>
       </c>
       <c r="D22">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E22">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F22">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G22">
         <v>0</v>
@@ -3173,13 +3173,13 @@
         <v>0</v>
       </c>
       <c r="L22">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="M22">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N22">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
@@ -3193,37 +3193,37 @@
         <v>75</v>
       </c>
       <c r="D23">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="E23">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="F23">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G23">
+        <v>215</v>
+      </c>
+      <c r="H23">
+        <v>3</v>
+      </c>
+      <c r="I23">
+        <v>18</v>
+      </c>
+      <c r="J23">
         <v>212</v>
       </c>
-      <c r="H23">
-        <v>7</v>
-      </c>
-      <c r="I23">
-        <v>12</v>
-      </c>
-      <c r="J23">
-        <v>205</v>
-      </c>
       <c r="K23">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="L23">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="M23">
         <v>9</v>
       </c>
       <c r="N23">
-        <v>230</v>
+        <v>239</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
@@ -3237,13 +3237,13 @@
         <v>74</v>
       </c>
       <c r="D24">
-        <v>519</v>
+        <v>497</v>
       </c>
       <c r="E24">
-        <v>474</v>
+        <v>451</v>
       </c>
       <c r="F24">
-        <v>474</v>
+        <v>451</v>
       </c>
       <c r="G24">
         <v>0</v>
@@ -3261,10 +3261,10 @@
         <v>0</v>
       </c>
       <c r="L24">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M24">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N24">
         <v>365</v>
@@ -3281,37 +3281,37 @@
         <v>75</v>
       </c>
       <c r="D25">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="E25">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="F25">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="G25">
-        <v>343</v>
+        <v>373</v>
       </c>
       <c r="H25">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I25">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="J25">
-        <v>325</v>
+        <v>360</v>
       </c>
       <c r="K25">
-        <v>325</v>
+        <v>360</v>
       </c>
       <c r="L25">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M25">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="N25">
-        <v>386</v>
+        <v>404</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
@@ -3325,13 +3325,13 @@
         <v>74</v>
       </c>
       <c r="D26">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="E26">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="F26">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -3349,13 +3349,13 @@
         <v>0</v>
       </c>
       <c r="L26">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="M26">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N26">
-        <v>208</v>
+        <v>225</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
@@ -3369,37 +3369,37 @@
         <v>75</v>
       </c>
       <c r="D27">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E27">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="F27">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="G27">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="H27">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I27">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J27">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="K27">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="L27">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="M27">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="N27">
-        <v>226</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -3408,7 +3408,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CB59B9A-3B10-441F-9DBF-88D23AAD34A8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6AA18B3-B337-4D95-87EA-58CF621CABE2}">
   <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3498,15 +3498,15 @@
       </c>
       <c r="C5" s="11">
         <f>Conteos!D4*Supuestos!$D$11+Conteos!E4*Supuestos!$D$12+Conteos!F4*Supuestos!$D$13+Conteos!G4*Supuestos!$D$14+Conteos!H4*Supuestos!$D$15+Conteos!I4*Supuestos!$D$16+Conteos!J4*Supuestos!$D$17</f>
-        <v>957</v>
+        <v>943.5</v>
       </c>
       <c r="D5" s="11">
         <f>Conteos!D5*Supuestos!$D$11+Conteos!E5*Supuestos!$D$12+Conteos!F5*Supuestos!$D$13+Conteos!G5*Supuestos!$D$14+Conteos!H5*Supuestos!$D$15+Conteos!I5*Supuestos!$D$16+Conteos!J5*Supuestos!$D$17</f>
-        <v>439</v>
+        <v>470.75</v>
       </c>
       <c r="E5" s="11">
         <f>C5-D5</f>
-        <v>518</v>
+        <v>472.75</v>
       </c>
       <c r="F5" s="9">
         <f>IF(B5="feria",E5*Supuestos!$D$8,0)</f>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="G5" s="9">
         <f>IF(B5="no feria",E5*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>101852.86403692825</v>
+        <v>92955.485469995809</v>
       </c>
       <c r="H5" s="9">
         <f>Conteos!K5*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3526,11 +3526,11 @@
       </c>
       <c r="J5" s="9">
         <f>F5+G5-H5-I5</f>
-        <v>89352.864036928251</v>
+        <v>80455.485469995809</v>
       </c>
       <c r="K5" s="9">
         <f>K4+J5</f>
-        <v>-910647.13596307172</v>
+        <v>-919544.51453000423</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -3544,19 +3544,19 @@
       </c>
       <c r="C6" s="11">
         <f>Conteos!D6*Supuestos!$D$11+Conteos!E6*Supuestos!$D$12+Conteos!F6*Supuestos!$D$13+Conteos!G6*Supuestos!$D$14+Conteos!H6*Supuestos!$D$15+Conteos!I6*Supuestos!$D$16+Conteos!J6*Supuestos!$D$17</f>
-        <v>1583</v>
+        <v>1608.5</v>
       </c>
       <c r="D6" s="11">
         <f>Conteos!D7*Supuestos!$D$11+Conteos!E7*Supuestos!$D$12+Conteos!F7*Supuestos!$D$13+Conteos!G7*Supuestos!$D$14+Conteos!H7*Supuestos!$D$15+Conteos!I7*Supuestos!$D$16+Conteos!J7*Supuestos!$D$17</f>
-        <v>746.25</v>
+        <v>793.5</v>
       </c>
       <c r="E6" s="11">
         <f>C6-D6</f>
-        <v>836.75</v>
+        <v>815</v>
       </c>
       <c r="F6" s="9">
         <f>IF(B6="feria",E6*Supuestos!$D$8,0)</f>
-        <v>164527.76830675619</v>
+        <v>160251.12778010912</v>
       </c>
       <c r="G6" s="9">
         <f>IF(B6="no feria",E6*Supuestos!$D$8*Supuestos!$D$24,0)</f>
@@ -3572,11 +3572,11 @@
       </c>
       <c r="J6" s="9">
         <f>F6+G6-H6-I6</f>
-        <v>152027.76830675619</v>
+        <v>147751.12778010912</v>
       </c>
       <c r="K6" s="9">
         <f>K5+J6</f>
-        <v>-758619.36765631556</v>
+        <v>-771793.38674989506</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -3590,15 +3590,15 @@
       </c>
       <c r="C7" s="11">
         <f>Conteos!D8*Supuestos!$D$11+Conteos!E8*Supuestos!$D$12+Conteos!F8*Supuestos!$D$13+Conteos!G8*Supuestos!$D$14+Conteos!H8*Supuestos!$D$15+Conteos!I8*Supuestos!$D$16+Conteos!J8*Supuestos!$D$17</f>
-        <v>955</v>
+        <v>1003</v>
       </c>
       <c r="D7" s="11">
         <f>Conteos!D9*Supuestos!$D$11+Conteos!E9*Supuestos!$D$12+Conteos!F9*Supuestos!$D$13+Conteos!G9*Supuestos!$D$14+Conteos!H9*Supuestos!$D$15+Conteos!I9*Supuestos!$D$16+Conteos!J9*Supuestos!$D$17</f>
-        <v>427.5</v>
+        <v>466.25</v>
       </c>
       <c r="E7" s="11">
         <f>C7-D7</f>
-        <v>527.5</v>
+        <v>536.75</v>
       </c>
       <c r="F7" s="9">
         <f>IF(B7="feria",E7*Supuestos!$D$8,0)</f>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="G7" s="9">
         <f>IF(B7="no feria",E7*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>103720.82196810743</v>
+        <v>105539.62311162401</v>
       </c>
       <c r="H7" s="9">
         <f>Conteos!K9*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3618,11 +3618,11 @@
       </c>
       <c r="J7" s="9">
         <f>F7+G7-H7-I7</f>
-        <v>91220.821968107426</v>
+        <v>93039.623111624009</v>
       </c>
       <c r="K7" s="9">
         <f>K6+J7</f>
-        <v>-667398.54568820819</v>
+        <v>-678753.76363827102</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -3636,15 +3636,15 @@
       </c>
       <c r="C8" s="11">
         <f>Conteos!D10*Supuestos!$D$11+Conteos!E10*Supuestos!$D$12+Conteos!F10*Supuestos!$D$13+Conteos!G10*Supuestos!$D$14+Conteos!H10*Supuestos!$D$15+Conteos!I10*Supuestos!$D$16+Conteos!J10*Supuestos!$D$17</f>
-        <v>971</v>
+        <v>917.5</v>
       </c>
       <c r="D8" s="11">
         <f>Conteos!D11*Supuestos!$D$11+Conteos!E11*Supuestos!$D$12+Conteos!F11*Supuestos!$D$13+Conteos!G11*Supuestos!$D$14+Conteos!H11*Supuestos!$D$15+Conteos!I11*Supuestos!$D$16+Conteos!J11*Supuestos!$D$17</f>
-        <v>497.5</v>
+        <v>430.75</v>
       </c>
       <c r="E8" s="11">
         <f>C8-D8</f>
-        <v>473.5</v>
+        <v>486.75</v>
       </c>
       <c r="F8" s="9">
         <f>IF(B8="feria",E8*Supuestos!$D$8,0)</f>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="G8" s="9">
         <f>IF(B8="no feria",E8*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>93102.955832983644</v>
+        <v>95708.265579101979</v>
       </c>
       <c r="H8" s="9">
         <f>Conteos!K11*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3664,11 +3664,11 @@
       </c>
       <c r="J8" s="9">
         <f>F8+G8-H8-I8</f>
-        <v>80602.955832983644</v>
+        <v>83208.265579101979</v>
       </c>
       <c r="K8" s="9">
         <f>K7+J8</f>
-        <v>-586795.58985522459</v>
+        <v>-595545.49805916904</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -3682,15 +3682,15 @@
       </c>
       <c r="C9" s="11">
         <f>Conteos!D12*Supuestos!$D$11+Conteos!E12*Supuestos!$D$12+Conteos!F12*Supuestos!$D$13+Conteos!G12*Supuestos!$D$14+Conteos!H12*Supuestos!$D$15+Conteos!I12*Supuestos!$D$16+Conteos!J12*Supuestos!$D$17</f>
-        <v>1019</v>
+        <v>1021.5</v>
       </c>
       <c r="D9" s="11">
         <f>Conteos!D13*Supuestos!$D$11+Conteos!E13*Supuestos!$D$12+Conteos!F13*Supuestos!$D$13+Conteos!G13*Supuestos!$D$14+Conteos!H13*Supuestos!$D$15+Conteos!I13*Supuestos!$D$16+Conteos!J13*Supuestos!$D$17</f>
-        <v>472.5</v>
+        <v>473</v>
       </c>
       <c r="E9" s="11">
         <f>C9-D9</f>
-        <v>546.5</v>
+        <v>548.5</v>
       </c>
       <c r="F9" s="9">
         <f>IF(B9="feria",E9*Supuestos!$D$8,0)</f>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="G9" s="9">
         <f>IF(B9="no feria",E9*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>107456.73783046581</v>
+        <v>107849.99213176669</v>
       </c>
       <c r="H9" s="9">
         <f>Conteos!K13*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3710,11 +3710,11 @@
       </c>
       <c r="J9" s="9">
         <f>F9+G9-H9-I9</f>
-        <v>94956.737830465805</v>
+        <v>95349.992131766689</v>
       </c>
       <c r="K9" s="9">
         <f>K8+J9</f>
-        <v>-491838.85202475882</v>
+        <v>-500195.50592740235</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -3728,15 +3728,15 @@
       </c>
       <c r="C10" s="11">
         <f>Conteos!D14*Supuestos!$D$11+Conteos!E14*Supuestos!$D$12+Conteos!F14*Supuestos!$D$13+Conteos!G14*Supuestos!$D$14+Conteos!H14*Supuestos!$D$15+Conteos!I14*Supuestos!$D$16+Conteos!J14*Supuestos!$D$17</f>
-        <v>810</v>
+        <v>945</v>
       </c>
       <c r="D10" s="11">
         <f>Conteos!D15*Supuestos!$D$11+Conteos!E15*Supuestos!$D$12+Conteos!F15*Supuestos!$D$13+Conteos!G15*Supuestos!$D$14+Conteos!H15*Supuestos!$D$15+Conteos!I15*Supuestos!$D$16+Conteos!J15*Supuestos!$D$17</f>
-        <v>420.25</v>
+        <v>454.5</v>
       </c>
       <c r="E10" s="11">
         <f>C10-D10</f>
-        <v>389.75</v>
+        <v>490.5</v>
       </c>
       <c r="F10" s="9">
         <f>IF(B10="feria",E10*Supuestos!$D$8,0)</f>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="G10" s="9">
         <f>IF(B10="no feria",E10*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>76635.43196600923</v>
+        <v>96445.617394041124</v>
       </c>
       <c r="H10" s="9">
         <f>Conteos!K15*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3756,11 +3756,11 @@
       </c>
       <c r="J10" s="9">
         <f>F10+G10-H10-I10</f>
-        <v>64135.43196600923</v>
+        <v>83945.617394041124</v>
       </c>
       <c r="K10" s="9">
         <f>K9+J10</f>
-        <v>-427703.42005874962</v>
+        <v>-416249.88853336126</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -3774,15 +3774,15 @@
       </c>
       <c r="C11" s="11">
         <f>Conteos!D16*Supuestos!$D$11+Conteos!E16*Supuestos!$D$12+Conteos!F16*Supuestos!$D$13+Conteos!G16*Supuestos!$D$14+Conteos!H16*Supuestos!$D$15+Conteos!I16*Supuestos!$D$16+Conteos!J16*Supuestos!$D$17</f>
-        <v>1068.5</v>
+        <v>1034.5</v>
       </c>
       <c r="D11" s="11">
         <f>Conteos!D17*Supuestos!$D$11+Conteos!E17*Supuestos!$D$12+Conteos!F17*Supuestos!$D$13+Conteos!G17*Supuestos!$D$14+Conteos!H17*Supuestos!$D$15+Conteos!I17*Supuestos!$D$16+Conteos!J17*Supuestos!$D$17</f>
-        <v>532.75</v>
+        <v>486.5</v>
       </c>
       <c r="E11" s="11">
         <f>C11-D11</f>
-        <v>535.75</v>
+        <v>548</v>
       </c>
       <c r="F11" s="9">
         <f>IF(B11="feria",E11*Supuestos!$D$8,0)</f>
@@ -3790,7 +3790,7 @@
       </c>
       <c r="G11" s="9">
         <f>IF(B11="no feria",E11*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>105342.99596097357</v>
+        <v>107751.67855644146</v>
       </c>
       <c r="H11" s="9">
         <f>Conteos!K17*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3802,11 +3802,11 @@
       </c>
       <c r="J11" s="9">
         <f>F11+G11-H11-I11</f>
-        <v>92842.995960973567</v>
+        <v>95251.67855644146</v>
       </c>
       <c r="K11" s="9">
         <f>K10+J11</f>
-        <v>-334860.42409777606</v>
+        <v>-320998.20997691981</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -3820,15 +3820,15 @@
       </c>
       <c r="C12" s="11">
         <f>Conteos!D18*Supuestos!$D$11+Conteos!E18*Supuestos!$D$12+Conteos!F18*Supuestos!$D$13+Conteos!G18*Supuestos!$D$14+Conteos!H18*Supuestos!$D$15+Conteos!I18*Supuestos!$D$16+Conteos!J18*Supuestos!$D$17</f>
-        <v>1018</v>
+        <v>1002</v>
       </c>
       <c r="D12" s="11">
         <f>Conteos!D19*Supuestos!$D$11+Conteos!E19*Supuestos!$D$12+Conteos!F19*Supuestos!$D$13+Conteos!G19*Supuestos!$D$14+Conteos!H19*Supuestos!$D$15+Conteos!I19*Supuestos!$D$16+Conteos!J19*Supuestos!$D$17</f>
-        <v>461.75</v>
+        <v>516.75</v>
       </c>
       <c r="E12" s="11">
         <f>C12-D12</f>
-        <v>556.25</v>
+        <v>485.25</v>
       </c>
       <c r="F12" s="9">
         <f>IF(B12="feria",E12*Supuestos!$D$8,0)</f>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="G12" s="9">
         <f>IF(B12="no feria",E12*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>109373.8525493076</v>
+        <v>95413.324853126309</v>
       </c>
       <c r="H12" s="9">
         <f>Conteos!K19*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3848,11 +3848,11 @@
       </c>
       <c r="J12" s="9">
         <f>F12+G12-H12-I12</f>
-        <v>96873.852549307601</v>
+        <v>82913.324853126309</v>
       </c>
       <c r="K12" s="9">
         <f>K11+J12</f>
-        <v>-237986.57154846846</v>
+        <v>-238084.8851237935</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -3866,15 +3866,15 @@
       </c>
       <c r="C13" s="11">
         <f>Conteos!D20*Supuestos!$D$11+Conteos!E20*Supuestos!$D$12+Conteos!F20*Supuestos!$D$13+Conteos!G20*Supuestos!$D$14+Conteos!H20*Supuestos!$D$15+Conteos!I20*Supuestos!$D$16+Conteos!J20*Supuestos!$D$17</f>
-        <v>1069.5</v>
+        <v>902</v>
       </c>
       <c r="D13" s="11">
         <f>Conteos!D21*Supuestos!$D$11+Conteos!E21*Supuestos!$D$12+Conteos!F21*Supuestos!$D$13+Conteos!G21*Supuestos!$D$14+Conteos!H21*Supuestos!$D$15+Conteos!I21*Supuestos!$D$16+Conteos!J21*Supuestos!$D$17</f>
-        <v>465</v>
+        <v>402.5</v>
       </c>
       <c r="E13" s="11">
         <f>C13-D13</f>
-        <v>604.5</v>
+        <v>499.5</v>
       </c>
       <c r="F13" s="9">
         <f>IF(B13="feria",E13*Supuestos!$D$8,0)</f>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="G13" s="9">
         <f>IF(B13="no feria",E13*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>118861.11256819135</v>
+        <v>98215.261749895086</v>
       </c>
       <c r="H13" s="9">
         <f>Conteos!K21*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3894,11 +3894,11 @@
       </c>
       <c r="J13" s="9">
         <f>F13+G13-H13-I13</f>
-        <v>106361.11256819135</v>
+        <v>85715.261749895086</v>
       </c>
       <c r="K13" s="9">
         <f>K12+J13</f>
-        <v>-131625.45898027712</v>
+        <v>-152369.62337389842</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -3912,15 +3912,15 @@
       </c>
       <c r="C14" s="11">
         <f>Conteos!D22*Supuestos!$D$11+Conteos!E22*Supuestos!$D$12+Conteos!F22*Supuestos!$D$13+Conteos!G22*Supuestos!$D$14+Conteos!H22*Supuestos!$D$15+Conteos!I22*Supuestos!$D$16+Conteos!J22*Supuestos!$D$17</f>
-        <v>1020</v>
+        <v>1025.5</v>
       </c>
       <c r="D14" s="11">
         <f>Conteos!D23*Supuestos!$D$11+Conteos!E23*Supuestos!$D$12+Conteos!F23*Supuestos!$D$13+Conteos!G23*Supuestos!$D$14+Conteos!H23*Supuestos!$D$15+Conteos!I23*Supuestos!$D$16+Conteos!J23*Supuestos!$D$17</f>
-        <v>431.25</v>
+        <v>475.75</v>
       </c>
       <c r="E14" s="11">
         <f>C14-D14</f>
-        <v>588.75</v>
+        <v>549.75</v>
       </c>
       <c r="F14" s="9">
         <f>IF(B14="feria",E14*Supuestos!$D$8,0)</f>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="G14" s="9">
         <f>IF(B14="no feria",E14*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>115764.23494544692</v>
+        <v>108095.77607007974</v>
       </c>
       <c r="H14" s="9">
         <f>Conteos!K23*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -3940,11 +3940,11 @@
       </c>
       <c r="J14" s="9">
         <f>F14+G14-H14-I14</f>
-        <v>103264.23494544692</v>
+        <v>95595.776070079737</v>
       </c>
       <c r="K14" s="9">
         <f>K13+J14</f>
-        <v>-28361.2240348302</v>
+        <v>-56773.847303818678</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -3958,19 +3958,19 @@
       </c>
       <c r="C15" s="11">
         <f>Conteos!D24*Supuestos!$D$11+Conteos!E24*Supuestos!$D$12+Conteos!F24*Supuestos!$D$13+Conteos!G24*Supuestos!$D$14+Conteos!H24*Supuestos!$D$15+Conteos!I24*Supuestos!$D$16+Conteos!J24*Supuestos!$D$17</f>
-        <v>1726.5</v>
+        <v>1647.5</v>
       </c>
       <c r="D15" s="11">
         <f>Conteos!D25*Supuestos!$D$11+Conteos!E25*Supuestos!$D$12+Conteos!F25*Supuestos!$D$13+Conteos!G25*Supuestos!$D$14+Conteos!H25*Supuestos!$D$15+Conteos!I25*Supuestos!$D$16+Conteos!J25*Supuestos!$D$17</f>
-        <v>775</v>
+        <v>753.75</v>
       </c>
       <c r="E15" s="11">
         <f>C15-D15</f>
-        <v>951.5</v>
+        <v>893.75</v>
       </c>
       <c r="F15" s="9">
         <f>IF(B15="feria",E15*Supuestos!$D$8,0)</f>
-        <v>187090.73384389427</v>
+        <v>175735.5158938313</v>
       </c>
       <c r="G15" s="9">
         <f>IF(B15="no feria",E15*Supuestos!$D$8*Supuestos!$D$24,0)</f>
@@ -3986,11 +3986,11 @@
       </c>
       <c r="J15" s="9">
         <f>F15+G15-H15-I15</f>
-        <v>174590.73384389427</v>
+        <v>163235.5158938313</v>
       </c>
       <c r="K15" s="9">
         <f>K14+J15</f>
-        <v>146229.50980906407</v>
+        <v>106461.66859001262</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
@@ -4004,15 +4004,15 @@
       </c>
       <c r="C16" s="11">
         <f>Conteos!D26*Supuestos!$D$11+Conteos!E26*Supuestos!$D$12+Conteos!F26*Supuestos!$D$13+Conteos!G26*Supuestos!$D$14+Conteos!H26*Supuestos!$D$15+Conteos!I26*Supuestos!$D$16+Conteos!J26*Supuestos!$D$17</f>
-        <v>918.5</v>
+        <v>955.5</v>
       </c>
       <c r="D16" s="11">
         <f>Conteos!D27*Supuestos!$D$11+Conteos!E27*Supuestos!$D$12+Conteos!F27*Supuestos!$D$13+Conteos!G27*Supuestos!$D$14+Conteos!H27*Supuestos!$D$15+Conteos!I27*Supuestos!$D$16+Conteos!J27*Supuestos!$D$17</f>
-        <v>460.5</v>
+        <v>456</v>
       </c>
       <c r="E16" s="11">
         <f>C16-D16</f>
-        <v>458</v>
+        <v>499.5</v>
       </c>
       <c r="F16" s="9">
         <f>IF(B16="feria",E16*Supuestos!$D$8,0)</f>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="G16" s="9">
         <f>IF(B16="no feria",E16*Supuestos!$D$8*Supuestos!$D$24,0)</f>
-        <v>90055.234997901804</v>
+        <v>98215.261749895086</v>
       </c>
       <c r="H16" s="9">
         <f>Conteos!K27*Supuestos!$D$19*Supuestos!$D$23</f>
@@ -4032,11 +4032,11 @@
       </c>
       <c r="J16" s="9">
         <f>F16+G16-H16-I16</f>
-        <v>77555.234997901804</v>
+        <v>85715.261749895086</v>
       </c>
       <c r="K16" s="9">
         <f>K15+J16</f>
-        <v>223784.74480696587</v>
+        <v>192176.9303399077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>